<commit_message>
30 Oct POEMS reconciliation: 36 lines + SGOV match to the cent; 9 NYSE marks set from POEMS; MV 874,941.02 ties; CAT order 7 sh LIMIT 647.39 / cap 653.86; workbook rebuilt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJZYTemDPd8XNBcdUBVnWw
</commit_message>
<xml_diff>
--- a/src/Pillar4_US_Portfolio_Workbook.xlsx
+++ b/src/Pillar4_US_Portfolio_Workbook.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oct 29, 2026 22:30 Bangkok - MSFT BOOKED 9 sh at 525.4031 = 4,738.75; cash 24,975.30. FULL POEMS RECONCILIATION: 36 lines + SGOV match to the cent; cash corrected by 0.10 (CRWD 19 Oct fee true-up); SGOV sale trued up to 10,047.25 (realised -27.25); October MONTHLY rebuilt (6 buys + 1 sale had been missing); October dividends 251.31 itemised. Prices: 54 names at the 28 Oct close, 9 at 27 Oct - the 29 Oct close is written by the next morning run. || PREVIOUS ENTRY: Oct 29, 2026 (03:30 UTC job) - DAILY PRICE REFRESH, 2nd pass: 11 more of the 15 stragglers resolved. Wed 2026-10-28 close written for ETN 392.88, GEV 878.03, PWR 606.89, COHR 239.59, SPCX 145.23, CIEN 363.21 (54 of 63 now at 10-28); verified Tue 10-27 close written for ARM 226.60, GE 297.66, MPWR 1211.89, LHX 259.40, TSEM 189.08 (marketbeat prev-close fields / heygotrade dated closes; every prev-close cross-checked against the stored prior close to the cent). Sources: 247wallst Oct-28 article sidebars validated to the cent on MSFT/ORCL/NVDA/MU/GOOGL/VRT; heygotrade dated close pages; stockanalysis/Google Finance/tipranks/marketscreener caches still frozen pre-close (4th night). 6%-movers vs last build, verified + allowed: PWR +7.6% (sidebar + 247wallst company page, prev 578.8x both), COHR +8.2% (sidebar; prev 235.79 = heygotrade 10-27 close exact), CIEN +8.1% (heygotrade 10-28 close 363.21 +3.43%; gurufocus +3.4% same evening). Unresolved, left at their verified 10-27 close: CDNS 343.08, CRDO 167.43, AVAV 126.73, CEG 258.98 (heygotrade 10-27 closes match the board to the cent; no readable 10-28 close). SPY 772.31 10-28 (marketchameleon dated close; SSGA official 10-27 769.66 added to risk_series with ycharts ust10 4.99 10-27; ust10 10-28 skipped - named sources not yet updated, fool.com wrap printed 5.02 at close for reference). HISTORY 10-28 row mv updated in place for the new ETN/GEV closes. || PREVIOUS ENTRY: Oct 29, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: 48 of 63 set to the Wed 2026-10-28 close (fool.com dated quote pages; stockanalysis/Google Finance/ycharts caches frozen pre-close for a third night). 15 unresolved stay at their prior close: holdings CDNS CRDO AVAV GEV ETN CEG (10-27), watch ARM MPWR COHR SPCX LHX PWR GE TSEM CIEN (10-26). QQQ 725.61 (10-28); SPY, spyHigh and risk_series spy/ust10 left unchanged - no clean close readable. HISTORY row 10-28 added. 6%-movers verified: ORCL 144.54 +10.73% d/d, VRT 242.94 +16.49% d/d, MU 983.23, SNDK 1404.77, STX 697.97 (247wallst sidebar matches to the cent); SNPS FN BE STRL on dated fool closes + headline corroboration. || PREVIOUS ENTRY: Oct 29, 2026 - GOOGL TEST APPROVED (Salee): 19 Nov $18,524 tranche moved to a 10 Dec DECIDE - buy only if no further share sale AND a credible path back to positive free cash flow; fail = budget cut to cost spent, no sale. || PREVIOUS ENTRY: Oct 29, 2026 04:45 Bangkok - RESULTS SCORED: MSFT PASS (BUY 9 sh tonight, limit 531.01, cap 536.32); STRL FAIL (signed backlog 4.14bn &lt; 4.33bn; budget back to pool; half 2 cancelled); GEV thesis intact (Power orders +178%, Electrification -9% on a tough comparison); VRT partial disclosure; GOOGL Q3 cloud doubled but FCF -9.1bn + June 84.75bn equity raise - 19 Nov tranche pending Salee. Fed held 3.75-4.00% (10-2, Cook and Hammack for a hike). SGOV 4 Nov sale no longer needed. || PREVIOUS ENTRY: Oct 28, 2026 - SGOV SLICE 1 BOOKED: SELL 100 at 100.6901 = 10,047.46 net (POEMS 1187938, 22:29 Bangkok). Cash 29,714.36; SGOV 694 sh parked (cost 69,917.06). || PREVIOUS ENTRY: Oct 28, 2026 13:16 Bangkok - PRICES OF THE 36 HOLDINGS SET TO THE TUE 2026-10-27 CLOSE FROM SALEE'S POEMS POSITIONS SCREEN (US market closed; POEMS "Current Price" column; SGOV mark 100.68). Reason: every web source reachable from the sandbox served pre-close cached pages for Oct 27 through both scheduled runs (00:30 and 03:30 UTC) and manual checks at 03:30-04:50 UTC, so 0 of 63 could be written by the job. The 27 watch names (no position) stay at the 26 Oct close until the next successful run. Moves of 6%+ vs 26 Oct: CDNS +6.5%, ALAB +10.5%, CRDO +10.8%, RKLB +8.3% - consistent with the reported 27 Oct session (AMD +5.5%, AVGO +4%, MU +2.8%, chips rally). Positions and cost on the same screen reconcile to the board to the cent on all 36 lines (641,827.76 NASD + 247,167.89 NYSE incl. SGOV = 888,995.64). pe/ps/fpe/peg/pfcf rescaled with price per the 26 Oct rule. || PREVIOUS ENTRY: Oct 28, 2026 (runs 00:30 + 03:30 UTC) - DAILY PRICE REFRESH: BOTH overnight passes could not resolve the Tue 2026-10-27 close for any ticker. 03:30 pass sampled 14 stockanalysis.com quote/history pages: every capture predated the 4:00 PM close (freshest stamps 10:05-11:25 AM EDT Oct 27; some caches as old as May 2025), and Google Finance (Sep 24/25 caches), marketscreener (Sep 4) and ycharts (Oct 26 18:04 EDT) were equally stale. Per the leave-unchanged rule nothing was written: all 63 prices, mcaps, P/E block, SPY/QQQ and pxd stay at the Mon 2026-10-26 close (CGNX still 2026-10-23); no HISTORY row; risk_series ust10/spy 10-27 skipped (sources unreadable; ust10 2026-10-26 = 5.00 was already added by the 00:30 pass). Oct-26 baseline cross-checked against 9 history tables - all matched. Every number checked came from a tool call this session; the next scheduled pass retries.</t>
+          <t>Oct 30, 2026 11:10 Bangkok - POEMS POSITIONS RECONCILED (screen 10:56 SGT, after the 29 Oct close): 36 lines + SGOV match to the cent; market value 874,941.02 ties. Nine NYSE marks set from POEMS (APH 82.08, ANET 184.22, CAT 647.39, ETN 393.72, TSM 431.81, VRT 245.92, V 410.54, VST 140.95; SGOV 100.71) - all within 0.2% of the job's closes; ratios rescaled. No fill tonight yet: CAT 7 sh LIMIT 647.39 (cap 653.86) is the only order. || PREVIOUS ENTRY: Oct 30, 2026 08:40 Bangkok - AMZN Q3 read recorded (AWS +39%, backlog $578bn, TTM FCF -$42.4bn, no order - over budget); CAT order set: 7 sh Day LIMIT 647.22, cap 653.69. || PREVIOUS ENTRY: Oct 30, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: all 63 prices set to the Thu 2026-10-29 close. Primary source this run: marketbeat.com dated daily-price tables / closing-price headers (pages updated 10/29, 'Closing price 4:00 PM Eastern' stamps), every ticker's prior close cross-checked against the stored board value; stockanalysis.com and Google Finance caches still frozen pre-close (5th night); GEV from the fool.com quote page previous-close field (887.85; method validated to the cent on GOOGL and MSFT this run). Big earnings-reaction day: 6%-movers verified + allowed: GOOGL 283.82 -12.64% (Q3 miss/FCF, fool prev-close field exact + news), FTNT 139.10 -20.09% (service-revenue forecast cut; 247wallst sidebar exact), MRVL 218.34 -13.24% (Lumentum deal talks; fool widget -13.24% exact), CAT 647.22 -9.49% (sales outlook; 247wallst sidebar 647.39), LHX 279.12 +7.10% (Q3 beat + raised FY guide; investing.com 278.65 +6.92%), AVAV 134.88 +7.09% (gurufocus +7.1%). SPY 769.36 and QQQ 715.34 (10-29, marketbeat closing headers; prev closes match board); spyHigh unchanged 779.09. risk_series spy 10-29 added; ust10 10-29 skipped (ycharts H15 only through 10-27; yahoo close bar printed 4.99 for reference). HISTORY 10-29 row added (first row including the 29 Oct MSFT buy, 126 sh). Note: TSEM 187.92 written from a dated 10/29 marketbeat header whose implied 10/28 prev close (193.52) could not be cross-checked - flagged for the next run. Every number from a tool call this session. || PREVIOUS ENTRY: Oct 29, 2026 23:00 Bangkok - GOOGL 10 Dec test (1) CLARIFIED: Q3 ATM share sales of $12.4bn were draws under the $40bn ATM announced in the June $84.75bn raise, so they do not fail the test; a new or upsized programme would. No order, budget or price changed. || PREVIOUS ENTRY: Oct 29, 2026 22:30 Bangkok - MSFT BOOKED 9 sh at 525.4031 = 4,738.75; cash 24,975.30. FULL POEMS RECONCILIATION: 36 lines + SGOV match to the cent; cash corrected by 0.10 (CRWD 19 Oct fee true-up); SGOV sale trued up to 10,047.25 (realised -27.25); October MONTHLY rebuilt (6 buys + 1 sale had been missing); October dividends 251.31 itemised. Prices: 54 names at the 28 Oct close, 9 at 27 Oct - the 29 Oct close is written by the next morning run. || PREVIOUS ENTRY: Oct 29, 2026 (03:30 UTC job) - DAILY PRICE REFRESH, 2nd pass: 11 more of the 15 stragglers resolved. Wed 2026-10-28 close written for ETN 392.88, GEV 878.03, PWR 606.89, COHR 239.59, SPCX 145.23, CIEN 363.21 (54 of 63 now at 10-28); verified Tue 10-27 close written for ARM 226.60, GE 297.66, MPWR 1211.89, LHX 259.40, TSEM 189.08 (marketbeat prev-close fields / heygotrade dated closes; every prev-close cross-checked against the stored prior close to the cent). Sources: 247wallst Oct-28 article sidebars validated to the cent on MSFT/ORCL/NVDA/MU/GOOGL/VRT; heygotrade dated close pages; stockanalysis/Google Finance/tipranks/marketscreener caches still frozen pre-close (4th night). 6%-movers vs last build, verified + allowed: PWR +7.6% (sidebar + 247wallst company page, prev 578.8x both), COHR +8.2% (sidebar; prev 235.79 = heygotrade 10-27 close exact), CIEN +8.1% (heygotrade 10-28 close 363.21 +3.43%; gurufocus +3.4% same evening). Unresolved, left at their verified 10-27 close: CDNS 343.08, CRDO 167.43, AVAV 126.73, CEG 258.98 (heygotrade 10-27 closes match the board to the cent; no readable 10-28 close). SPY 772.31 10-28 (marketchameleon dated close; SSGA official 10-27 769.66 added to risk_series with ycharts ust10 4.99 10-27; ust10 10-28 skipped - named sources not yet updated, fool.com wrap printed 5.02 at close for reference). HISTORY 10-28 row mv updated in place for the new ETN/GEV closes. || PREVIOUS ENTRY: Oct 29, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: 48 of 63 set to the Wed 2026-10-28 close (fool.com dated quote pages; stockanalysis/Google Finance/ycharts caches frozen pre-close for a third night). 15 unresolved stay at their prior close: holdings CDNS CRDO AVAV GEV ETN CEG (10-27), watch ARM MPWR COHR SPCX LHX PWR GE TSEM CIEN (10-26). QQQ 725.61 (10-28); SPY, spyHigh and risk_series spy/ust10 left unchanged - no clean close readable. HISTORY row 10-28 added. 6%-movers verified: ORCL 144.54 +10.73% d/d, VRT 242.94 +16.49% d/d, MU 983.23, SNDK 1404.77, STX 697.97 (247wallst sidebar matches to the cent); SNPS FN BE STRL on dated fool closes + headline corroboration. || PREVIOUS ENTRY: Oct 29, 2026 - GOOGL TEST APPROVED (Salee): 19 Nov $18,524 tranche moved to a 10 Dec DECIDE - buy only if no further share sale AND a credible path back to positive free cash flow; fail = budget cut to cost spent, no sale. || PREVIOUS ENTRY: Oct 29, 2026 04:45 Bangkok - RESULTS SCORED: MSFT PASS (BUY 9 sh tonight, limit 531.01, cap 536.32); STRL FAIL (signed backlog 4.14bn &lt; 4.33bn; budget back to pool; half 2 cancelled); GEV thesis intact (Power orders +178%, Electrification -9% on a tough comparison); VRT partial disclosure; GOOGL Q3 cloud doubled but FCF -9.1bn + June 84.75bn equity raise - 19 Nov tranche pending Salee. Fed held 3.75-4.00% (10-2, Cook and Hammack for a hike). SGOV 4 Nov sale no longer needed. || PREVIOUS ENTRY: Oct 28, 2026 - SGOV SLICE 1 BOOKED: SELL 100 at 100.6901 = 10,047.46 net (POEMS 1187938, 22:29 Bangkok). Cash 29,714.36; SGOV 694 sh parked (cost 69,917.06). || PREVIOUS ENTRY: Oct 28, 2026 13:16 Bangkok - PRICES OF THE 36 HOLDINGS SET TO THE TUE 2026-10-27 CLOSE FROM SALEE'S POEMS POSITIONS SCREEN (US market closed; POEMS "Current Price" column; SGOV mark 100.68). Reason: every web source reachable from the sandbox served pre-close cached pages for Oct 27 through both scheduled runs (00:30 and 03:30 UTC) and manual checks at 03:30-04:50 UTC, so 0 of 63 could be written by the job. The 27 watch names (no position) stay at the 26 Oct close until the next successful run. Moves of 6%+ vs 26 Oct: CDNS +6.5%, ALAB +10.5%, CRDO +10.8%, RKLB +8.3% - consistent with the reported 27 Oct session (AMD +5.5%, AVGO +4%, MU +2.8%, chips rally). Positions and cost on the same screen reconcile to the board to the cent on all 36 lines (641,827.76 NASD + 247,167.89 NYSE incl. SGOV = 888,995.64). pe/ps/fpe/peg/pfcf rescaled with price per the 26 Oct rule. || PREVIOUS ENTRY: Oct 28, 2026 (runs 00:30 + 03:30 UTC) - DAILY PRICE REFRESH: BOTH overnight passes could not resolve the Tue 2026-10-27 close for any ticker. 03:30 pass sampled 14 stockanalysis.com quote/history pages: every capture predated the 4:00 PM close (freshest stamps 10:05-11:25 AM EDT Oct 27; some caches as old as May 2025), and Google Finance (Sep 24/25 caches), marketscreener (Sep 4) and ycharts (Oct 26 18:04 EDT) were equally stale. Per the leave-unchanged rule nothing was written: all 63 prices, mcaps, P/E block, SPY/QQQ and pxd stay at the Mon 2026-10-26 close (CGNX still 2026-10-23); no HISTORY row; risk_series ust10/spy 10-27 skipped (sources unreadable; ust10 2026-10-26 = 5.00 was already added by the 00:30 pass). Oct-26 baseline cross-checked against 9 history tables - all matched. Every number checked came from a tool call this session; the next scheduled pass retries.</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>823805.88</v>
+        <v>805048.28</v>
       </c>
     </row>
     <row r="6">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>100092.47</v>
+        <v>81334.87</v>
       </c>
     </row>
     <row r="7">
@@ -517,7 +517,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>+13.83%</t>
+          <t>+11.24%</t>
         </is>
       </c>
     </row>
@@ -675,16 +675,16 @@
         <v>274.0825806451613</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>324.89</v>
+        <v>283.82</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>70501.12999999999</v>
+        <v>61588.94</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>11025.20999999999</v>
+        <v>2113.019999999997</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.1853726684681799</v>
+        <v>0.03552731929157207</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>32.2446</v>
@@ -693,7 +693,7 @@
         <v>1917777.250032</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>2372363.024499999</v>
+        <v>2072467.831</v>
       </c>
     </row>
     <row r="3">
@@ -722,16 +722,16 @@
         <v>457.2834126984127</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>531.01</v>
+        <v>530.14</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>66907.25999999999</v>
+        <v>66797.64</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>9289.549999999996</v>
+        <v>9179.93</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.1612273379139851</v>
+        <v>0.1593247978789855</v>
       </c>
       <c r="K3" s="3" t="n">
         <v>32.0119</v>
@@ -740,7 +740,7 @@
         <v>1844452.370749</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>2251429.299</v>
+        <v>2247740.586</v>
       </c>
     </row>
     <row r="4">
@@ -769,16 +769,16 @@
         <v>232.5394736842105</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>254.6</v>
+        <v>243.79</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>53211.4</v>
+        <v>50952.11</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>4610.650000000001</v>
+        <v>2351.360000000001</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.09486787755332997</v>
+        <v>0.04838114638148589</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>32.3066</v>
@@ -787,7 +787,7 @@
         <v>1570124.98995</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>1790563.61</v>
+        <v>1714538.5015</v>
       </c>
     </row>
     <row r="5">
@@ -816,16 +816,16 @@
         <v>659.6042580645161</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>612.49</v>
+        <v>624.52</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>47467.975</v>
+        <v>48400.3</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-3651.355000000003</v>
+        <v>-2719.030000000006</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.07142806840386999</v>
+        <v>-0.05318985988274897</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>32.2596</v>
@@ -834,7 +834,7 @@
         <v>1649089.138068</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>1597297.35875</v>
+        <v>1628670.095</v>
       </c>
     </row>
     <row r="6">
@@ -863,16 +863,16 @@
         <v>190.9340707964602</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>215.38</v>
+        <v>213.66</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>97351.75999999999</v>
+        <v>96574.31999999999</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>11049.56</v>
+        <v>10272.12</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.1280333525680689</v>
+        <v>0.1190250074737376</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>32.084</v>
@@ -881,7 +881,7 @@
         <v>2768919.7848</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>3275886.723999999</v>
+        <v>3249725.868</v>
       </c>
     </row>
     <row r="7">
@@ -910,16 +910,16 @@
         <v>340.3975141242938</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>351.81</v>
+        <v>345</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>31135.185</v>
+        <v>30532.5</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>1010.005000000001</v>
+        <v>407.3199999999997</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.03352693660253651</v>
+        <v>0.01352091506175232</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>31.6503</v>
@@ -928,7 +928,7 @@
         <v>953470.9845540001</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1047698.97525</v>
+        <v>1027418.625</v>
       </c>
     </row>
     <row r="8">
@@ -957,16 +957,16 @@
         <v>250.7130909090909</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>578.4400000000001</v>
+        <v>566.42</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>31814.2</v>
+        <v>31153.1</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>18024.98</v>
+        <v>17363.88</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>1.30717908627174</v>
+        <v>1.259235837850146</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>32.0515</v>
@@ -975,7 +975,7 @@
         <v>441965.1848299999</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>1070547.83</v>
+        <v>1048301.815</v>
       </c>
     </row>
     <row r="9">
@@ -1004,16 +1004,16 @@
         <v>215.550890052356</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>251.65</v>
+        <v>218.34</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>24032.575</v>
+        <v>20851.47</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>3447.465</v>
+        <v>266.3600000000006</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.1674737225110772</v>
+        <v>0.01293944992278402</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>32.5019</v>
@@ -1022,7 +1022,7 @@
         <v>669055.186709</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>808696.1487499999</v>
+        <v>701651.9655</v>
       </c>
     </row>
     <row r="10">
@@ -1051,16 +1051,16 @@
         <v>326.5008333333333</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>343.08</v>
+        <v>342.75</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>4116.96</v>
+        <v>4113</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>198.9499999999998</v>
+        <v>194.9899999999998</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.05077832879446448</v>
+        <v>0.04976761161916375</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>32.32</v>
@@ -1069,7 +1069,7 @@
         <v>126630.0832</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>138535.704</v>
+        <v>138402.45</v>
       </c>
     </row>
     <row r="11">
@@ -1098,16 +1098,16 @@
         <v>378.1683870967742</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>439.51</v>
+        <v>431.81</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>74936.455</v>
+        <v>73623.605</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>10458.745</v>
+        <v>9145.894999999997</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.1622071410414545</v>
+        <v>0.1418458409890797</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>31.9974</v>
@@ -1116,7 +1116,7 @@
         <v>2063119.077954</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>2521611.71075</v>
+        <v>2477434.30825</v>
       </c>
     </row>
     <row r="12">
@@ -1145,16 +1145,16 @@
         <v>1345.164705882353</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>1662.85</v>
+        <v>1675.7</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>28268.45</v>
+        <v>28486.9</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>5400.649999999998</v>
+        <v>5619.100000000002</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.2361683240189261</v>
+        <v>0.2457210575569142</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>32.372</v>
@@ -1163,7 +1163,7 @@
         <v>740276.4216</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>951233.3424999999</v>
+        <v>958584.1850000001</v>
       </c>
     </row>
     <row r="13">
@@ -1192,16 +1192,16 @@
         <v>186.3690909090909</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>253.82</v>
+        <v>254.39</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>5584.04</v>
+        <v>5596.58</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>1483.92</v>
+        <v>1496.46</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.3619211145039657</v>
+        <v>0.3649795615738076</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>31.4491</v>
@@ -1210,7 +1210,7 @@
         <v>128945.083892</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>187902.946</v>
+        <v>188324.917</v>
       </c>
     </row>
     <row r="14">
@@ -1239,16 +1239,16 @@
         <v>345.6519298245614</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>416</v>
+        <v>421.66</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>23712</v>
+        <v>24034.62</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4009.84</v>
+        <v>4332.460000000003</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.2035228624678715</v>
+        <v>0.2198977167985643</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>32.1085</v>
@@ -1257,7 +1257,7 @@
         <v>632606.80436</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>797908.7999999999</v>
+        <v>808764.9630000001</v>
       </c>
     </row>
     <row r="15">
@@ -1286,16 +1286,16 @@
         <v>195.0383333333333</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>158.77</v>
+        <v>167.43</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>2857.86</v>
+        <v>3013.74</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-652.8299999999999</v>
+        <v>-496.9499999999998</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.1859548977551421</v>
+        <v>-0.1415533698503712</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>32.1216</v>
@@ -1304,7 +1304,7 @@
         <v>112768.979904</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>96166.989</v>
+        <v>101412.351</v>
       </c>
     </row>
     <row r="16">
@@ -1333,16 +1333,16 @@
         <v>356.737</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>313.24</v>
+        <v>296.23</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>3132.4</v>
+        <v>2962.3</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-434.9699999999998</v>
+        <v>-605.0699999999997</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.1219301614354552</v>
+        <v>-0.1696123474716667</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>32.6972</v>
@@ -1351,7 +1351,7 @@
         <v>116643.010364</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>105405.26</v>
+        <v>99681.395</v>
       </c>
     </row>
     <row r="17">
@@ -1380,16 +1380,16 @@
         <v>753.9935288169869</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>983.23</v>
+        <v>934.27</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>48620.7235</v>
+        <v>46199.6515</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>11335.7435</v>
+        <v>8914.671499999997</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.3040297594366417</v>
+        <v>0.2390955151377309</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>32.1376</v>
@@ -1398,7 +1398,7 @@
         <v>1198249.773248</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>1636087.345775</v>
+        <v>1554618.272975</v>
       </c>
     </row>
     <row r="18">
@@ -1427,16 +1427,16 @@
         <v>159.0364285714286</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>186.72</v>
+        <v>184.22</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>18298.56</v>
+        <v>18053.56</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>2712.990000000002</v>
+        <v>2467.990000000002</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.1740706307180297</v>
+        <v>0.15835096181917</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>32.6011</v>
@@ -1445,7 +1445,7 @@
         <v>508106.726127</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>615746.544</v>
+        <v>607502.294</v>
       </c>
     </row>
     <row r="19">
@@ -1474,16 +1474,16 @@
         <v>79.426</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>80.95999999999999</v>
+        <v>82.08</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>8500.799999999999</v>
+        <v>8618.4</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>161.0699999999997</v>
+        <v>278.6700000000001</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.0193135748999068</v>
+        <v>0.03341475083725733</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>32.34</v>
@@ -1492,7 +1492,7 @@
         <v>269706.8682</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>286051.92</v>
+        <v>290009.16</v>
       </c>
     </row>
     <row r="20">
@@ -1521,16 +1521,16 @@
         <v>815.0208695652174</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>913.95</v>
+        <v>919.53</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>10510.425</v>
+        <v>10574.595</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>1137.685000000001</v>
+        <v>1201.855</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.1213823278998459</v>
+        <v>0.1282287783508344</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>32.5803</v>
@@ -1539,7 +1539,7 @@
         <v>305366.681022</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>353675.80125</v>
+        <v>355835.12175</v>
       </c>
     </row>
     <row r="21">
@@ -1568,16 +1568,16 @@
         <v>253.698</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>297.2</v>
+        <v>290.43</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>4458</v>
+        <v>4356.45</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>652.5300000000002</v>
+        <v>550.98</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.1714715922080585</v>
+        <v>0.1447863207435613</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>32.4697</v>
@@ -1586,7 +1586,7 @@
         <v>123562.469259</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>150011.7</v>
+        <v>146594.5425</v>
       </c>
     </row>
     <row r="22">
@@ -1615,16 +1615,16 @@
         <v>157.2364864864865</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>167.43</v>
+        <v>165.29</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>18584.73</v>
+        <v>18347.19</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>1131.48</v>
+        <v>893.9399999999987</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.06482918654118858</v>
+        <v>0.05121911391861107</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>32.4342</v>
@@ -1633,7 +1633,7 @@
         <v>566082.20115</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>625376.1645</v>
+        <v>617382.9434999999</v>
       </c>
     </row>
     <row r="23">
@@ -1662,16 +1662,16 @@
         <v>200.356</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>176.3</v>
+        <v>176.89</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1763</v>
+        <v>1768.9</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>-240.5599999999999</v>
+        <v>-234.6600000000001</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.1200662820180079</v>
+        <v>-0.1171215236878357</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>33.65</v>
@@ -1680,7 +1680,7 @@
         <v>67419.79399999999</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>59324.95</v>
+        <v>59523.48499999999</v>
       </c>
     </row>
     <row r="24">
@@ -1709,16 +1709,16 @@
         <v>65.60677419354839</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>58.43</v>
+        <v>58.97</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>3622.66</v>
+        <v>3656.14</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-444.96</v>
+        <v>-411.48</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>-0.1093907493817023</v>
+        <v>-0.1011598920253121</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>33.0687</v>
@@ -1727,7 +1727,7 @@
         <v>134510.905494</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>121902.509</v>
+        <v>123029.111</v>
       </c>
     </row>
     <row r="25">
@@ -1756,16 +1756,16 @@
         <v>84.45999999999999</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>58.6</v>
+        <v>59.1</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1347.8</v>
+        <v>1359.3</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-594.78</v>
+        <v>-583.28</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>-0.3061804404451812</v>
+        <v>-0.3002604783329387</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>33.31</v>
@@ -1774,7 +1774,7 @@
         <v>64707.3398</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>45353.46999999999</v>
+        <v>45740.445</v>
       </c>
     </row>
     <row r="26">
@@ -1803,16 +1803,16 @@
         <v>138.32725</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>196.81</v>
+        <v>196.42</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>7872.4</v>
+        <v>7856.799999999999</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>2339.309999999999</v>
+        <v>2323.709999999999</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.422785459842511</v>
+        <v>0.4199660587483665</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>31.79</v>
@@ -1821,7 +1821,7 @@
         <v>175896.9311</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>264906.26</v>
+        <v>264381.3199999999</v>
       </c>
     </row>
     <row r="27">
@@ -1850,16 +1850,16 @@
         <v>208.7944444444445</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>126.73</v>
+        <v>134.88</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>2281.14</v>
+        <v>2427.84</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-1477.16</v>
+        <v>-1330.46</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>-0.3930394061144667</v>
+        <v>-0.3540058004949046</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>32.3497</v>
@@ -1868,7 +1868,7 @@
         <v>121579.87751</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>76760.36099999999</v>
+        <v>81696.81600000001</v>
       </c>
     </row>
     <row r="28">
@@ -1897,16 +1897,16 @@
         <v>431.0968421052632</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>444.18</v>
+        <v>448.76</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>16878.84</v>
+        <v>17052.88</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>497.1599999999999</v>
+        <v>671.2000000000007</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.03034853568132205</v>
+        <v>0.04097259865898984</v>
       </c>
       <c r="K28" s="3" t="n">
         <v>32.1878</v>
@@ -1915,7 +1915,7 @@
         <v>527290.2395040001</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>567972.966</v>
+        <v>573829.412</v>
       </c>
     </row>
     <row r="29">
@@ -1944,16 +1944,16 @@
         <v>376.0583333333333</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>400.6</v>
+        <v>410.54</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>7210.8</v>
+        <v>7389.72</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>441.75</v>
+        <v>620.6700000000001</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.06526026547299843</v>
+        <v>0.0916923349657633</v>
       </c>
       <c r="K29" s="3" t="n">
         <v>33.65</v>
@@ -1962,7 +1962,7 @@
         <v>227778.5325</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>242643.42</v>
+        <v>248664.078</v>
       </c>
     </row>
     <row r="30">
@@ -1991,16 +1991,16 @@
         <v>249.8636842105263</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>394.49</v>
+        <v>380.57</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>14990.62</v>
+        <v>14461.66</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>5495.800000000001</v>
+        <v>4966.84</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.5788208728548832</v>
+        <v>0.5231104960388928</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>32.5467</v>
@@ -2009,7 +2009,7 @@
         <v>309025.058094</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>504434.363</v>
+        <v>486634.859</v>
       </c>
     </row>
     <row r="31">
@@ -2038,16 +2038,16 @@
         <v>960.0600000000001</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>878.03</v>
+        <v>887.85</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>11414.39</v>
+        <v>11542.05</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-1066.390000000001</v>
+        <v>-938.7299999999996</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>-0.08544257650563516</v>
+        <v>-0.07521404912192985</v>
       </c>
       <c r="K31" s="3" t="n">
         <v>32.66</v>
@@ -2056,7 +2056,7 @@
         <v>407622.2748</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>384094.2235</v>
+        <v>388389.9825</v>
       </c>
     </row>
     <row r="32">
@@ -2085,16 +2085,16 @@
         <v>418.511923076923</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>392.88</v>
+        <v>393.72</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>10214.88</v>
+        <v>10236.72</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-666.4300000000003</v>
+        <v>-644.5899999999983</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>-0.0612453831386111</v>
+        <v>-0.05923827186248699</v>
       </c>
       <c r="K32" s="3" t="n">
         <v>32.3317</v>
@@ -2103,7 +2103,7 @@
         <v>351811.2505269999</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>343730.7119999999</v>
+        <v>344465.628</v>
       </c>
     </row>
     <row r="33">
@@ -2132,16 +2132,16 @@
         <v>246.5205952380952</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>242.94</v>
+        <v>245.92</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>20406.96</v>
+        <v>20657.28</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>-300.7700000000004</v>
+        <v>-50.45000000000073</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>-0.01452452779710767</v>
+        <v>-0.002436288284616456</v>
       </c>
       <c r="K33" s="3" t="n">
         <v>31.4889</v>
@@ -2150,7 +2150,7 @@
         <v>652063.639197</v>
       </c>
       <c r="M33" s="6" t="n">
-        <v>686694.2039999999</v>
+        <v>695117.472</v>
       </c>
     </row>
     <row r="34">
@@ -2179,16 +2179,16 @@
         <v>263.88640625</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>258.98</v>
+        <v>264.58</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>16574.72</v>
+        <v>16933.12</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>-314.0099999999984</v>
+        <v>44.38999999999942</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>-0.0185928722882063</v>
+        <v>0.002628379990680141</v>
       </c>
       <c r="K34" s="3" t="n">
         <v>33.0112</v>
@@ -2197,7 +2197,7 @@
         <v>557517.243776</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>557739.328</v>
+        <v>569799.4879999999</v>
       </c>
     </row>
     <row r="35">
@@ -2226,16 +2226,16 @@
         <v>140.3488679245283</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>142.72</v>
+        <v>140.95</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>15128.32</v>
+        <v>14940.7</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>251.3400000000001</v>
+        <v>63.71999999999935</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>0.0168945579008643</v>
+        <v>0.004283127355148649</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>32.9329</v>
@@ -2244,7 +2244,7 @@
         <v>489942.0946419999</v>
       </c>
       <c r="M35" s="6" t="n">
-        <v>509067.968</v>
+        <v>502754.5549999999</v>
       </c>
     </row>
     <row r="36">
@@ -2273,16 +2273,16 @@
         <v>248.6436956521739</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>343.83</v>
+        <v>348.91</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>15816.18</v>
+        <v>16049.86</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>4378.569999999998</v>
+        <v>4612.25</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.3828221105633081</v>
+        <v>0.4032529523213328</v>
       </c>
       <c r="K36" s="3" t="n">
         <v>32.4331</v>
@@ -2291,7 +2291,7 @@
         <v>370957.1488910001</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>532214.4569999999</v>
+        <v>540077.789</v>
       </c>
     </row>
     <row r="37">
@@ -2320,16 +2320,16 @@
         <v>814.7583333333333</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>713.38</v>
+        <v>647.39</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>4280.28</v>
+        <v>3884.34</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-608.2700000000004</v>
+        <v>-1004.21</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>-0.1244274887236503</v>
+        <v>-0.2054208303075554</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>33.65</v>
@@ -2338,7 +2338,7 @@
         <v>164499.7075</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>144031.422</v>
+        <v>130708.041</v>
       </c>
     </row>
     <row r="38">
@@ -2351,13 +2351,13 @@
         <v>723713.41</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>823805.8785</v>
+        <v>805048.2814999999</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>100092.4685</v>
+        <v>81334.87149999989</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>0.138304012495775</v>
+        <v>0.112385469684747</v>
       </c>
     </row>
   </sheetData>
@@ -2552,22 +2552,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>324.89</v>
+        <v>283.82</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3977.5387</v>
+        <v>3474.73</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>16.97</v>
+        <v>14.82</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>24.29</v>
+        <v>21.22</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>8.44</v>
+        <v>7.38</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1.82</v>
+        <v>1.59</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>60.86</v>
@@ -2618,7 +2618,7 @@
         <v>26.4</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>201.39</v>
+        <v>175.93</v>
       </c>
       <c r="Z2" s="3" t="n">
         <v>21.91</v>
@@ -2639,19 +2639,19 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>531.01</v>
+        <v>530.14</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>3955.4014</v>
+        <v>3948.9209</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>27.73</v>
+        <v>27.68</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.87</v>
+        <v>26.83</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>11.42</v>
+        <v>11.4</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>1.69</v>
@@ -2705,7 +2705,7 @@
         <v>35.2</v>
       </c>
       <c r="Y3" s="3" t="n">
-        <v>65.97</v>
+        <v>65.86</v>
       </c>
       <c r="Z3" s="3" t="n">
         <v>20.32</v>
@@ -2726,22 +2726,22 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>254.6</v>
+        <v>243.79</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2746.806</v>
+        <v>2630.18</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>29.57</v>
+        <v>28.31</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27.1</v>
+        <v>25.95</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3.54</v>
+        <v>3.39</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.31</v>
+        <v>1.25</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>50.77</v>
@@ -2810,22 +2810,22 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>612.49</v>
+        <v>624.52</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1564.3526</v>
+        <v>1595.0783</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>20.89</v>
+        <v>21.3</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>18.6</v>
+        <v>18.97</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>6.47</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>81.03</v>
@@ -2876,7 +2876,7 @@
         <v>37.9</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>54.64</v>
+        <v>55.71</v>
       </c>
       <c r="Z5" s="3" t="n">
         <v>14.42</v>
@@ -2897,19 +2897,19 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>215.38</v>
+        <v>213.66</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5214.246</v>
+        <v>5172.6056</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>27.23</v>
+        <v>27.01</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>17.81</v>
+        <v>17.67</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>17.21</v>
+        <v>17.07</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>0.36</v>
@@ -2963,7 +2963,7 @@
         <v>125.3</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>40.95</v>
+        <v>40.62</v>
       </c>
       <c r="Z6" s="3" t="n">
         <v>25.19</v>
@@ -2984,22 +2984,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>351.81</v>
+        <v>345</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1671.9296</v>
+        <v>1639.566</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>44.87</v>
+        <v>44.01</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>20.26</v>
+        <v>19.87</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>18.76</v>
+        <v>18.4</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>68.77</v>
@@ -3050,7 +3050,7 @@
         <v>92.90000000000001</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>42.62</v>
+        <v>41.8</v>
       </c>
       <c r="Z7" s="3" t="n">
         <v>30.06</v>
@@ -3071,22 +3071,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>578.4400000000001</v>
+        <v>566.42</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>944.2895</v>
+        <v>924.6671</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>148.7</v>
+        <v>145.61</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>52.04</v>
+        <v>50.96</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>22.86</v>
+        <v>22.39</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>53.06</v>
@@ -3137,7 +3137,7 @@
         <v>61.3</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>112.38</v>
+        <v>110.04</v>
       </c>
       <c r="Z8" s="3" t="n">
         <v>87.31</v>
@@ -3158,22 +3158,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>226.6</v>
+        <v>228.77</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>242.0311</v>
+        <v>244.3489</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>231.22</v>
+        <v>233.44</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>94.88</v>
+        <v>95.79000000000001</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>46.91</v>
+        <v>47.35</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3.12</v>
+        <v>3.15</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>97.54000000000001</v>
@@ -3224,7 +3224,7 @@
         <v>54.3</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>160.7</v>
+        <v>162.24</v>
       </c>
       <c r="Z9" s="3" t="n">
         <v>208</v>
@@ -3245,22 +3245,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>251.65</v>
+        <v>218.34</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>220.3848</v>
+        <v>191.2133</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>83.88</v>
+        <v>72.78</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>44.53</v>
+        <v>38.64</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>23.32</v>
+        <v>20.23</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>53.1</v>
@@ -3308,7 +3308,7 @@
         <v>49.1</v>
       </c>
       <c r="Y10" s="3" t="n">
-        <v>127.55</v>
+        <v>110.67</v>
       </c>
       <c r="Z10" s="3" t="n">
         <v>70.78</v>
@@ -3329,19 +3329,19 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>343.08</v>
+        <v>342.75</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>94.601</v>
+        <v>94.51000000000001</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>68.20999999999999</v>
+        <v>68.14</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>39.88</v>
+        <v>39.84</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>15.43</v>
+        <v>15.42</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>2.64</v>
@@ -3395,7 +3395,7 @@
         <v>46.4</v>
       </c>
       <c r="Y11" s="3" t="n">
-        <v>53.58</v>
+        <v>53.53</v>
       </c>
       <c r="Z11" s="3" t="n">
         <v>40.27</v>
@@ -3416,22 +3416,22 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>481.89</v>
+        <v>490.19</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>92.274</v>
+        <v>93.8633</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>85.14</v>
+        <v>86.61</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27.28</v>
+        <v>27.75</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>72.59999999999999</v>
@@ -3482,7 +3482,7 @@
         <v>75.40000000000001</v>
       </c>
       <c r="Y12" s="3" t="n">
-        <v>33.61</v>
+        <v>34.19</v>
       </c>
       <c r="Z12" s="3" t="n">
         <v>43.2</v>
@@ -3503,22 +3503,22 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1211.89</v>
+        <v>1198.81</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>59.5595</v>
+        <v>58.9167</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>73.94</v>
+        <v>73.14</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>37.5</v>
+        <v>37.1</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>18.21</v>
+        <v>18.02</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>55.2</v>
@@ -3569,7 +3569,7 @@
         <v>47.9</v>
       </c>
       <c r="Y13" s="3" t="n">
-        <v>101.71</v>
+        <v>100.61</v>
       </c>
       <c r="Z13" s="3" t="n">
         <v>54.62</v>
@@ -3590,19 +3590,19 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>439.51</v>
+        <v>431.81</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>2120.0832</v>
+        <v>2082.9404</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>29.07</v>
+        <v>28.56</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>20.58</v>
+        <v>20.22</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>13.84</v>
+        <v>13.6</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>65.83</v>
@@ -3653,7 +3653,7 @@
         <v>66.09999999999999</v>
       </c>
       <c r="Y14" s="3" t="n">
-        <v>43.82</v>
+        <v>42.99</v>
       </c>
       <c r="Z14" s="3" t="n">
         <v>15.87</v>
@@ -3674,19 +3674,19 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1662.85</v>
+        <v>1675.7</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>649.347</v>
+        <v>654.365</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>42.38</v>
+        <v>42.7</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>26.17</v>
+        <v>26.37</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>14.69</v>
+        <v>14.8</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>54.34</v>
@@ -3737,7 +3737,7 @@
         <v>48.5</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>26.97</v>
+        <v>27.18</v>
       </c>
       <c r="Z15" s="3" t="n">
         <v>32.17</v>
@@ -3758,19 +3758,19 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>253.82</v>
+        <v>254.39</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>317.6002</v>
+        <v>318.3134</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>37.83</v>
+        <v>37.91</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.7</v>
+        <v>24.76</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>12.15</v>
+        <v>12.18</v>
       </c>
       <c r="H16" s="3" t="n">
         <v>0.89</v>
@@ -3824,7 +3824,7 @@
         <v>58.4</v>
       </c>
       <c r="Y16" s="3" t="n">
-        <v>48.5</v>
+        <v>48.61</v>
       </c>
       <c r="Z16" s="3" t="n">
         <v>28.05</v>
@@ -3845,22 +3845,22 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>416</v>
+        <v>421.66</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>330.2892</v>
+        <v>334.783</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>35.86</v>
+        <v>36.35</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23.59</v>
+        <v>23.91</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>10.71</v>
+        <v>10.86</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>50.3</v>
@@ -3911,7 +3911,7 @@
         <v>26</v>
       </c>
       <c r="Y17" s="3" t="n">
-        <v>58.71</v>
+        <v>59.51</v>
       </c>
       <c r="Z17" s="3" t="n">
         <v>29.29</v>
@@ -3932,22 +3932,22 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>158.77</v>
+        <v>167.43</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>207.3959</v>
+        <v>218.7082</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>39.79</v>
+        <v>41.96</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>29.06</v>
+        <v>30.65</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>14.29</v>
+        <v>15.07</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1.44</v>
+        <v>1.52</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>61.3</v>
@@ -3998,7 +3998,7 @@
         <v>43.6</v>
       </c>
       <c r="Y18" s="3" t="n">
-        <v>51.34</v>
+        <v>54.14</v>
       </c>
       <c r="Z18" s="3" t="n">
         <v>31.59</v>
@@ -4019,22 +4019,22 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>313.24</v>
+        <v>296.23</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>49.3324</v>
+        <v>46.6535</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>35.96</v>
+        <v>34.01</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>33.59</v>
+        <v>31.77</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>9.869999999999999</v>
+        <v>9.33</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>59.3</v>
@@ -4085,7 +4085,7 @@
         <v>95.3</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>48.37</v>
+        <v>45.74</v>
       </c>
       <c r="Z19" s="3" t="n">
         <v>31.81</v>
@@ -4106,19 +4106,19 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>983.23</v>
+        <v>934.27</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1110.4512</v>
+        <v>1055.1562</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>13.23</v>
+        <v>12.57</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>5.57</v>
+        <v>5.29</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>8.34</v>
+        <v>7.92</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -4172,7 +4172,7 @@
         <v>300.6</v>
       </c>
       <c r="Y20" s="3" t="n">
-        <v>18.87</v>
+        <v>17.93</v>
       </c>
       <c r="Z20" s="3" t="n">
         <v>8.49</v>
@@ -4193,22 +4193,22 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1404.77</v>
+        <v>1330.05</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>208.0273</v>
+        <v>196.9623</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>19.05</v>
+        <v>18.03</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>6.53</v>
+        <v>6.18</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>10.27</v>
+        <v>9.73</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>71.47</v>
@@ -4256,7 +4256,7 @@
         <v>232.1</v>
       </c>
       <c r="Y21" s="3" t="n">
-        <v>17.89</v>
+        <v>16.94</v>
       </c>
       <c r="Z21" s="3" t="n">
         <v>13.86</v>
@@ -4277,19 +4277,19 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>697.97</v>
+        <v>700.47</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>157.9263</v>
+        <v>158.492</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>36.62</v>
+        <v>36.75</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>19.98</v>
+        <v>20.05</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>11.44</v>
+        <v>11.48</v>
       </c>
       <c r="H22" s="3" t="n">
         <v>0.25</v>
@@ -4343,7 +4343,7 @@
         <v>74.5</v>
       </c>
       <c r="Y22" s="3" t="n">
-        <v>37.96</v>
+        <v>38.1</v>
       </c>
       <c r="Z22" s="3" t="n">
         <v>32.33</v>
@@ -4364,22 +4364,22 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>186.72</v>
+        <v>184.22</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>233.5895</v>
+        <v>230.462</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>59.09</v>
+        <v>58.3</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>40.15</v>
+        <v>39.61</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>22.16</v>
+        <v>21.86</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>63.54</v>
@@ -4430,7 +4430,7 @@
         <v>81.5</v>
       </c>
       <c r="Y23" s="3" t="n">
-        <v>45.68</v>
+        <v>45.04</v>
       </c>
       <c r="Z23" s="3" t="n">
         <v>43.98</v>
@@ -4448,22 +4448,22 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>80.95999999999999</v>
+        <v>82.08</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>199.6492</v>
+        <v>202.4112</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>29.23</v>
+        <v>29.63</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.21</v>
+        <v>27.58</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>6.04</v>
+        <v>6.13</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>1.38</v>
+        <v>1.4</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>38.81</v>
@@ -4514,7 +4514,7 @@
         <v>73.09999999999999</v>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>38.84</v>
+        <v>39.46</v>
       </c>
       <c r="Z24" s="3" t="n">
         <v>20.72</v>
@@ -4535,22 +4535,22 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>131.2</v>
+        <v>128.87</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>113.0194</v>
+        <v>111.0123</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>53.55</v>
+        <v>52.6</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>34.89</v>
+        <v>34.27</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>6.38</v>
+        <v>6.26</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1.09</v>
+        <v>1.07</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>36.5</v>
@@ -4601,7 +4601,7 @@
         <v>32.7</v>
       </c>
       <c r="Y25" s="3" t="n">
-        <v>45.76</v>
+        <v>44.95</v>
       </c>
       <c r="Z25" s="3" t="n">
         <v>27.77</v>
@@ -4622,16 +4622,16 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>913.95</v>
+        <v>919.53</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>71.0989</v>
+        <v>71.533</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>41.95</v>
+        <v>42.21</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>23.62</v>
+        <v>23.77</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>0.36</v>
@@ -4682,7 +4682,7 @@
         <v>93.2</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>275.86</v>
+        <v>277.54</v>
       </c>
       <c r="Z26" s="3" t="n">
         <v>84.20999999999999</v>
@@ -4703,22 +4703,22 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>239.59</v>
+        <v>236.9</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46.8699</v>
+        <v>46.3437</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>58.15</v>
+        <v>57.5</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>25.53</v>
+        <v>25.24</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>6.58</v>
+        <v>6.51</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>37.5</v>
@@ -4784,22 +4784,22 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>297.2</v>
+        <v>290.43</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>50.9421</v>
+        <v>49.7817</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>168.86</v>
+        <v>165.02</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>52.9</v>
+        <v>51.69</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>42.45</v>
+        <v>41.48</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>75.98999999999999</v>
@@ -4850,7 +4850,7 @@
         <v>121.5</v>
       </c>
       <c r="Y28" s="3" t="n">
-        <v>186.35</v>
+        <v>182.11</v>
       </c>
       <c r="Z28" s="3" t="n">
         <v>152.09</v>
@@ -4871,22 +4871,22 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>167.43</v>
+        <v>165.29</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>31.2238</v>
+        <v>30.8247</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>58.95</v>
+        <v>58.2</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>22.95</v>
+        <v>22.66</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>19.64</v>
+        <v>19.39</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.45</v>
+        <v>0.44</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>67.06999999999999</v>
@@ -4937,7 +4937,7 @@
         <v>190.7</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>71.75</v>
+        <v>70.83</v>
       </c>
       <c r="Z29" s="3" t="n">
         <v>49.6</v>
@@ -4958,19 +4958,19 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>367.3</v>
+        <v>349.15</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>13.1636</v>
+        <v>12.5131</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>28.15</v>
+        <v>26.75</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>20.14</v>
+        <v>19.14</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>2.84</v>
+        <v>2.7</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>12</v>
@@ -5039,19 +5039,19 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>176.3</v>
+        <v>176.89</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>18.9802</v>
+        <v>19.0437</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>10.87</v>
+        <v>10.91</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>8.369999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>3.53</v>
+        <v>3.54</v>
       </c>
       <c r="H31" s="3" t="n">
         <v>0.48</v>
@@ -5105,7 +5105,7 @@
         <v>51.7</v>
       </c>
       <c r="Y31" s="3" t="n">
-        <v>12.62</v>
+        <v>12.66</v>
       </c>
       <c r="Z31" s="3" t="n">
         <v>7.1</v>
@@ -5126,19 +5126,19 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>58.43</v>
+        <v>58.97</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>9.729699999999999</v>
+        <v>9.819599999999999</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>56.73</v>
+        <v>57.25</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>32.57</v>
+        <v>32.87</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>8.93</v>
+        <v>9.02</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>68.87</v>
@@ -5189,7 +5189,7 @@
         <v>39.3</v>
       </c>
       <c r="Y32" s="3" t="n">
-        <v>36.63</v>
+        <v>36.97</v>
       </c>
       <c r="Z32" s="3" t="n">
         <v>33.71</v>
@@ -5210,16 +5210,16 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>145.23</v>
+        <v>143.89</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>1970.7681</v>
+        <v>1952.5843</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>51.52</v>
+        <v>51.04</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>61.51</v>
+        <v>60.94</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>51.87</v>
@@ -5276,13 +5276,13 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>58.6</v>
+        <v>59.1</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>35.0696</v>
+        <v>35.3688</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>45.6</v>
+        <v>45.98</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>37.27</v>
@@ -5345,19 +5345,19 @@
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>196.81</v>
+        <v>196.42</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>471.8115</v>
+        <v>470.8766</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>168.21</v>
+        <v>167.88</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>103.44</v>
+        <v>103.24</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>76.72</v>
+        <v>76.56999999999999</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>1.94</v>
@@ -5411,7 +5411,7 @@
         <v>133.1</v>
       </c>
       <c r="Y35" s="3" t="n">
-        <v>140.84</v>
+        <v>140.56</v>
       </c>
       <c r="Z35" s="3" t="n">
         <v>174.12</v>
@@ -5432,22 +5432,22 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>259.4</v>
+        <v>279.12</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>48.3042</v>
+        <v>51.9764</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>26.2</v>
+        <v>28.19</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>20.6</v>
+        <v>22.17</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>2.11</v>
+        <v>2.27</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1.24</v>
+        <v>1.33</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>25.48</v>
@@ -5492,7 +5492,7 @@
         <v>19.5</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>17.2</v>
+        <v>18.51</v>
       </c>
       <c r="Z36" s="3" t="n">
         <v>13.71</v>
@@ -5513,19 +5513,19 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>41.17</v>
+        <v>43.59</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>7.7268</v>
+        <v>8.180999999999999</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>242.18</v>
+        <v>256.41</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>43.49</v>
+        <v>46.05</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>5.08</v>
+        <v>5.38</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>23</v>
@@ -5594,19 +5594,19 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>126.73</v>
+        <v>134.88</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>6.3852</v>
+        <v>6.7958</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>37.79</v>
+        <v>40.22</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>3.19</v>
+        <v>3.4</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>1.12</v>
+        <v>1.19</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>26.47</v>
@@ -5672,22 +5672,22 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>278.41</v>
+        <v>265.84</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>99.0817</v>
+        <v>94.6082</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>556.8200000000001</v>
+        <v>531.6799999999999</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>104.99</v>
+        <v>100.25</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>24.96</v>
+        <v>23.83</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>4.23</v>
+        <v>4.04</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>79.53</v>
@@ -5738,7 +5738,7 @@
         <v>61.3</v>
       </c>
       <c r="Y39" s="3" t="n">
-        <v>84.56999999999999</v>
+        <v>80.75</v>
       </c>
       <c r="AA39" s="3" t="n">
         <v>0.29</v>
@@ -5756,22 +5756,22 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>444.18</v>
+        <v>448.76</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>156.9141</v>
+        <v>158.5321</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>53.71</v>
+        <v>54.26</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>36.87</v>
+        <v>37.25</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>13.55</v>
+        <v>13.69</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>2.36</v>
+        <v>2.38</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>67.19</v>
@@ -5822,7 +5822,7 @@
         <v>48.3</v>
       </c>
       <c r="Y40" s="3" t="n">
-        <v>42.81</v>
+        <v>43.25</v>
       </c>
       <c r="Z40" s="3" t="n">
         <v>34.16</v>
@@ -5840,22 +5840,22 @@
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>144.54</v>
+        <v>139.51</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>437.0538</v>
+        <v>421.8443</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>22.66</v>
+        <v>21.87</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>16.98</v>
+        <v>16.39</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>6.09</v>
+        <v>5.88</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>63.96</v>
@@ -5924,22 +5924,22 @@
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>400.6</v>
+        <v>410.54</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>735.3484</v>
+        <v>753.5944</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>32.52</v>
+        <v>33.32</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>27.49</v>
+        <v>28.17</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>16.02</v>
+        <v>16.42</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>1.9</v>
+        <v>1.95</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>80.18000000000001</v>
@@ -5990,7 +5990,7 @@
         <v>60.92</v>
       </c>
       <c r="Y42" s="3" t="n">
-        <v>34.7</v>
+        <v>35.54</v>
       </c>
       <c r="Z42" s="3" t="n">
         <v>24.4</v>
@@ -6011,19 +6011,19 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>91.43000000000001</v>
+        <v>91.59</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>82.3216</v>
+        <v>82.4657</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>42.33</v>
+        <v>42.4</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>36.78</v>
+        <v>36.84</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>16.21</v>
+        <v>16.23</v>
       </c>
       <c r="H43" s="3" t="n">
         <v>1.77</v>
@@ -6077,7 +6077,7 @@
         <v>80.2</v>
       </c>
       <c r="Y43" s="3" t="n">
-        <v>27.26</v>
+        <v>27.31</v>
       </c>
       <c r="Z43" s="3" t="n">
         <v>29.41</v>
@@ -6098,22 +6098,22 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>394.49</v>
+        <v>380.57</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>322.69</v>
+        <v>311.3035</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>986.23</v>
+        <v>951.42</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>94.12</v>
+        <v>90.8</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>28.11</v>
+        <v>27.12</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>5.02</v>
+        <v>4.84</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>70.36</v>
@@ -6164,7 +6164,7 @@
         <v>60.3</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>78.45999999999999</v>
+        <v>75.69</v>
       </c>
       <c r="Z44" s="3" t="n">
         <v>199.22</v>
@@ -6185,22 +6185,22 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>266.66</v>
+        <v>261.15</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>273.6274</v>
+        <v>267.9734</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>6666.5</v>
+        <v>6528.75</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>188.76</v>
+        <v>184.86</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>50.77</v>
+        <v>49.72</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>6.44</v>
+        <v>6.31</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>75.14</v>
@@ -6248,7 +6248,7 @@
         <v>52.5</v>
       </c>
       <c r="Y45" s="3" t="n">
-        <v>170.09</v>
+        <v>166.58</v>
       </c>
       <c r="AA45" s="3" t="n">
         <v>0.16</v>
@@ -6266,22 +6266,22 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>174.08</v>
+        <v>139.1</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>127.5335</v>
+        <v>101.9067</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>56.7</v>
+        <v>45.31</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>49.58</v>
+        <v>39.62</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>16.18</v>
+        <v>12.93</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>3.03</v>
+        <v>2.42</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>79.75</v>
@@ -6332,7 +6332,7 @@
         <v>63.8</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>37.18</v>
+        <v>29.71</v>
       </c>
       <c r="Z46" s="3" t="n">
         <v>49.52</v>
@@ -6353,19 +6353,19 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>318.72</v>
+        <v>310.04</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>113.1309</v>
+        <v>110.0499</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>215.18</v>
+        <v>209.32</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>45.07</v>
+        <v>43.84</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>4.32</v>
+        <v>4.2</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>72.58</v>
@@ -6413,7 +6413,7 @@
         <v>47.2</v>
       </c>
       <c r="Y47" s="3" t="n">
-        <v>331.92</v>
+        <v>322.88</v>
       </c>
       <c r="AA47" s="3" t="n">
         <v>2.18</v>
@@ -6431,22 +6431,22 @@
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>134.96</v>
+        <v>137.98</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>12.4871</v>
+        <v>12.7665</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>34.96</v>
+        <v>35.75</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>27.08</v>
+        <v>27.69</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>3.56</v>
+        <v>3.64</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>2.04</v>
+        <v>2.09</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>22.08</v>
@@ -6497,7 +6497,7 @@
         <v>32.8</v>
       </c>
       <c r="Y48" s="3" t="n">
-        <v>39.04</v>
+        <v>39.91</v>
       </c>
       <c r="Z48" s="3" t="n">
         <v>27.42</v>
@@ -6518,22 +6518,22 @@
         </is>
       </c>
       <c r="C49" s="3" t="n">
-        <v>878.03</v>
+        <v>887.85</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>233.8452</v>
+        <v>236.4606</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>22.99</v>
+        <v>23.24</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>41.8</v>
+        <v>42.27</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>5.31</v>
+        <v>5.37</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="I49" s="3" t="n">
         <v>20.57</v>
@@ -6584,7 +6584,7 @@
         <v>55.8</v>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>13.67</v>
+        <v>13.82</v>
       </c>
       <c r="Z49" s="3" t="n">
         <v>52.98</v>
@@ -6605,19 +6605,19 @@
         </is>
       </c>
       <c r="C50" s="3" t="n">
-        <v>392.88</v>
+        <v>393.72</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>152.5509</v>
+        <v>152.877</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>40.01</v>
+        <v>40.09</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>25.93</v>
+        <v>25.98</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>5.08</v>
+        <v>5.09</v>
       </c>
       <c r="H50" s="3" t="n">
         <v>1.97</v>
@@ -6671,7 +6671,7 @@
         <v>28.7</v>
       </c>
       <c r="Y50" s="3" t="n">
-        <v>38.79</v>
+        <v>38.81</v>
       </c>
       <c r="Z50" s="3" t="n">
         <v>24.53</v>
@@ -6692,22 +6692,22 @@
         </is>
       </c>
       <c r="C51" s="3" t="n">
-        <v>242.94</v>
+        <v>245.92</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>93.5283</v>
+        <v>94.6756</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>45.41</v>
+        <v>45.96</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>30.67</v>
+        <v>31.05</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>7.13</v>
+        <v>7.21</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="I51" s="3" t="n">
         <v>38.12</v>
@@ -6758,7 +6758,7 @@
         <v>59.3</v>
       </c>
       <c r="Y51" s="3" t="n">
-        <v>29.69</v>
+        <v>30.08</v>
       </c>
       <c r="Z51" s="3" t="n">
         <v>28.01</v>
@@ -6779,22 +6779,22 @@
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>606.89</v>
+        <v>632.79</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>91.2436</v>
+        <v>95.13760000000001</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>69.44</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>32.65</v>
+        <v>34.04</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>2.77</v>
+        <v>2.89</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>1.57</v>
+        <v>1.64</v>
       </c>
       <c r="I52" s="3" t="n">
         <v>15.46</v>
@@ -6845,7 +6845,7 @@
         <v>33.25</v>
       </c>
       <c r="Y52" s="3" t="n">
-        <v>39.88</v>
+        <v>41.58</v>
       </c>
       <c r="Z52" s="3" t="n">
         <v>28.98</v>
@@ -6866,22 +6866,22 @@
         </is>
       </c>
       <c r="C53" s="3" t="n">
-        <v>228.08</v>
+        <v>222.28</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>67.17449999999999</v>
+        <v>65.4663</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>132.6</v>
+        <v>129.23</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>47.09</v>
+        <v>45.89</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>17.54</v>
+        <v>17.09</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="I53" s="3" t="n">
         <v>32.66</v>
@@ -6929,7 +6929,7 @@
         <v>122</v>
       </c>
       <c r="Y53" s="3" t="n">
-        <v>154.42</v>
+        <v>150.49</v>
       </c>
       <c r="Z53" s="3" t="n">
         <v>95.28</v>
@@ -6950,22 +6950,22 @@
         </is>
       </c>
       <c r="C54" s="3" t="n">
-        <v>258.98</v>
+        <v>264.58</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>92.4802</v>
+        <v>94.4799</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>25.07</v>
+        <v>25.61</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>20.94</v>
+        <v>21.39</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>2.96</v>
+        <v>3.02</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="I54" s="3" t="n">
         <v>22.11</v>
@@ -7016,7 +7016,7 @@
         <v>26.9</v>
       </c>
       <c r="Y54" s="3" t="n">
-        <v>311.05</v>
+        <v>317.78</v>
       </c>
       <c r="Z54" s="3" t="n">
         <v>14.31</v>
@@ -7037,22 +7037,22 @@
         </is>
       </c>
       <c r="C55" s="3" t="n">
-        <v>142.72</v>
+        <v>140.95</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>48.1226</v>
+        <v>47.5258</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>24.31</v>
+        <v>24.01</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>14.07</v>
+        <v>13.89</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>2.51</v>
+        <v>2.48</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="I55" s="3" t="n">
         <v>38.31</v>
@@ -7103,7 +7103,7 @@
         <v>15.5</v>
       </c>
       <c r="Y55" s="3" t="n">
-        <v>21.23</v>
+        <v>20.92</v>
       </c>
       <c r="Z55" s="3" t="n">
         <v>10.1</v>
@@ -7124,22 +7124,22 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>343.83</v>
+        <v>348.91</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>5019.825</v>
+        <v>5093.9916</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>39.25</v>
+        <v>39.83</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>37.5</v>
+        <v>38.05</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>10.75</v>
+        <v>10.91</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>3.38</v>
+        <v>3.43</v>
       </c>
       <c r="I56" s="3" t="n">
         <v>48.65</v>
@@ -7190,7 +7190,7 @@
         <v>45.64</v>
       </c>
       <c r="Y56" s="3" t="n">
-        <v>36.71</v>
+        <v>37.25</v>
       </c>
       <c r="Z56" s="3" t="n">
         <v>29.84</v>
@@ -7211,19 +7211,19 @@
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>61.99</v>
+        <v>62.05</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>258.1186</v>
+        <v>258.3684</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>17.97</v>
+        <v>17.99</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>17.27</v>
+        <v>17.29</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>5.19</v>
+        <v>5.2</v>
       </c>
       <c r="H57" s="3" t="n">
         <v>0.82</v>
@@ -7277,7 +7277,7 @@
         <v>34.7</v>
       </c>
       <c r="Y57" s="3" t="n">
-        <v>22.38</v>
+        <v>22.4</v>
       </c>
       <c r="Z57" s="3" t="n">
         <v>17.53</v>
@@ -7298,22 +7298,22 @@
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>259.97</v>
+        <v>254.91</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>87.3373</v>
+        <v>85.6374</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>19.98</v>
+        <v>19.59</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>14.47</v>
+        <v>14.19</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>12.79</v>
+        <v>12.54</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="I58" s="3" t="n">
         <v>88.45999999999999</v>
@@ -7361,7 +7361,7 @@
         <v>126.9</v>
       </c>
       <c r="Y58" s="3" t="n">
-        <v>19.22</v>
+        <v>18.85</v>
       </c>
       <c r="Z58" s="3" t="n">
         <v>16.17</v>
@@ -7382,22 +7382,22 @@
         </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>75.18000000000001</v>
+        <v>76.58</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46.0482</v>
+        <v>46.9057</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>29.03</v>
+        <v>29.57</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>17.66</v>
+        <v>17.99</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>1.66</v>
+        <v>1.69</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="I59" s="3" t="n">
         <v>44.34</v>
@@ -7448,7 +7448,7 @@
         <v>60</v>
       </c>
       <c r="Y59" s="3" t="n">
-        <v>10.95</v>
+        <v>11.15</v>
       </c>
       <c r="Z59" s="3" t="n">
         <v>15.18</v>
@@ -7469,22 +7469,22 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>713.38</v>
+        <v>647.39</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>327.9197</v>
+        <v>297.586</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>30.74</v>
+        <v>27.9</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>24.61</v>
+        <v>22.34</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>4.39</v>
+        <v>3.98</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>1.34</v>
+        <v>1.22</v>
       </c>
       <c r="I60" s="3" t="n">
         <v>29.71</v>
@@ -7535,7 +7535,7 @@
         <v>30.4</v>
       </c>
       <c r="Y60" s="3" t="n">
-        <v>36.45</v>
+        <v>33.07</v>
       </c>
       <c r="Z60" s="3" t="n">
         <v>21.84</v>
@@ -7556,22 +7556,22 @@
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>297.66</v>
+        <v>313.28</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>308.8402</v>
+        <v>325.0469</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>34.33</v>
+        <v>36.13</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>33.5</v>
+        <v>35.26</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>5.87</v>
+        <v>6.18</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>2.14</v>
+        <v>2.25</v>
       </c>
       <c r="I61" s="3" t="n">
         <v>30.07</v>
@@ -7622,7 +7622,7 @@
         <v>34.9</v>
       </c>
       <c r="Y61" s="3" t="n">
-        <v>38.36</v>
+        <v>40.37</v>
       </c>
       <c r="Z61" s="3" t="n">
         <v>26.34</v>
@@ -7643,22 +7643,22 @@
         </is>
       </c>
       <c r="C62" s="3" t="n">
-        <v>388.87</v>
+        <v>373.66</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>11.8924</v>
+        <v>11.4272</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>21.82</v>
+        <v>20.97</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>17.32</v>
+        <v>16.64</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>2.76</v>
+        <v>2.65</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
       <c r="I62" s="3" t="n">
         <v>23.78</v>
@@ -7709,7 +7709,7 @@
         <v>104.1</v>
       </c>
       <c r="Y62" s="3" t="n">
-        <v>25.25</v>
+        <v>24.26</v>
       </c>
       <c r="Z62" s="3" t="n">
         <v>15.04</v>
@@ -7730,22 +7730,22 @@
         </is>
       </c>
       <c r="C63" s="3" t="n">
-        <v>189.08</v>
+        <v>187.92</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>21.3732</v>
+        <v>21.2421</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>74.73999999999999</v>
+        <v>74.28</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>36.63</v>
+        <v>36.41</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>12.5</v>
+        <v>12.42</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="I63" s="3" t="n">
         <v>26.87</v>
@@ -7793,7 +7793,7 @@
         <v>32.5</v>
       </c>
       <c r="Y63" s="3" t="n">
-        <v>71.40000000000001</v>
+        <v>70.95999999999999</v>
       </c>
       <c r="Z63" s="3" t="n">
         <v>29.62</v>
@@ -7814,22 +7814,22 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>363.21</v>
+        <v>348.57</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>51.5086</v>
+        <v>49.4324</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>81.26000000000001</v>
+        <v>77.98</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>34.9</v>
+        <v>33.49</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>8.550000000000001</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="I64" s="3" t="n">
         <v>44.07</v>
@@ -7865,7 +7865,7 @@
         <v>46.1</v>
       </c>
       <c r="Y64" s="3" t="n">
-        <v>63.25</v>
+        <v>60.7</v>
       </c>
       <c r="Z64" s="3" t="n">
         <v>44.72</v>

</xml_diff>

<commit_message>
30 Oct: CAT BUY 7 @ 633.5642 = 4,444.44 booked (13 sh, cost 9,332.99); cash 20,530.86; MONTHLY Oct + investedEver updated; workbook rebuilt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJZYTemDPd8XNBcdUBVnWw
</commit_message>
<xml_diff>
--- a/src/Pillar4_US_Portfolio_Workbook.xlsx
+++ b/src/Pillar4_US_Portfolio_Workbook.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oct 30, 2026 11:10 Bangkok - POEMS POSITIONS RECONCILED (screen 10:56 SGT, after the 29 Oct close): 36 lines + SGOV match to the cent; market value 874,941.02 ties. Nine NYSE marks set from POEMS (APH 82.08, ANET 184.22, CAT 647.39, ETN 393.72, TSM 431.81, VRT 245.92, V 410.54, VST 140.95; SGOV 100.71) - all within 0.2% of the job's closes; ratios rescaled. No fill tonight yet: CAT 7 sh LIMIT 647.39 (cap 653.86) is the only order. || PREVIOUS ENTRY: Oct 30, 2026 08:40 Bangkok - AMZN Q3 read recorded (AWS +39%, backlog $578bn, TTM FCF -$42.4bn, no order - over budget); CAT order set: 7 sh Day LIMIT 647.22, cap 653.69. || PREVIOUS ENTRY: Oct 30, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: all 63 prices set to the Thu 2026-10-29 close. Primary source this run: marketbeat.com dated daily-price tables / closing-price headers (pages updated 10/29, 'Closing price 4:00 PM Eastern' stamps), every ticker's prior close cross-checked against the stored board value; stockanalysis.com and Google Finance caches still frozen pre-close (5th night); GEV from the fool.com quote page previous-close field (887.85; method validated to the cent on GOOGL and MSFT this run). Big earnings-reaction day: 6%-movers verified + allowed: GOOGL 283.82 -12.64% (Q3 miss/FCF, fool prev-close field exact + news), FTNT 139.10 -20.09% (service-revenue forecast cut; 247wallst sidebar exact), MRVL 218.34 -13.24% (Lumentum deal talks; fool widget -13.24% exact), CAT 647.22 -9.49% (sales outlook; 247wallst sidebar 647.39), LHX 279.12 +7.10% (Q3 beat + raised FY guide; investing.com 278.65 +6.92%), AVAV 134.88 +7.09% (gurufocus +7.1%). SPY 769.36 and QQQ 715.34 (10-29, marketbeat closing headers; prev closes match board); spyHigh unchanged 779.09. risk_series spy 10-29 added; ust10 10-29 skipped (ycharts H15 only through 10-27; yahoo close bar printed 4.99 for reference). HISTORY 10-29 row added (first row including the 29 Oct MSFT buy, 126 sh). Note: TSEM 187.92 written from a dated 10/29 marketbeat header whose implied 10/28 prev close (193.52) could not be cross-checked - flagged for the next run. Every number from a tool call this session. || PREVIOUS ENTRY: Oct 29, 2026 23:00 Bangkok - GOOGL 10 Dec test (1) CLARIFIED: Q3 ATM share sales of $12.4bn were draws under the $40bn ATM announced in the June $84.75bn raise, so they do not fail the test; a new or upsized programme would. No order, budget or price changed. || PREVIOUS ENTRY: Oct 29, 2026 22:30 Bangkok - MSFT BOOKED 9 sh at 525.4031 = 4,738.75; cash 24,975.30. FULL POEMS RECONCILIATION: 36 lines + SGOV match to the cent; cash corrected by 0.10 (CRWD 19 Oct fee true-up); SGOV sale trued up to 10,047.25 (realised -27.25); October MONTHLY rebuilt (6 buys + 1 sale had been missing); October dividends 251.31 itemised. Prices: 54 names at the 28 Oct close, 9 at 27 Oct - the 29 Oct close is written by the next morning run. || PREVIOUS ENTRY: Oct 29, 2026 (03:30 UTC job) - DAILY PRICE REFRESH, 2nd pass: 11 more of the 15 stragglers resolved. Wed 2026-10-28 close written for ETN 392.88, GEV 878.03, PWR 606.89, COHR 239.59, SPCX 145.23, CIEN 363.21 (54 of 63 now at 10-28); verified Tue 10-27 close written for ARM 226.60, GE 297.66, MPWR 1211.89, LHX 259.40, TSEM 189.08 (marketbeat prev-close fields / heygotrade dated closes; every prev-close cross-checked against the stored prior close to the cent). Sources: 247wallst Oct-28 article sidebars validated to the cent on MSFT/ORCL/NVDA/MU/GOOGL/VRT; heygotrade dated close pages; stockanalysis/Google Finance/tipranks/marketscreener caches still frozen pre-close (4th night). 6%-movers vs last build, verified + allowed: PWR +7.6% (sidebar + 247wallst company page, prev 578.8x both), COHR +8.2% (sidebar; prev 235.79 = heygotrade 10-27 close exact), CIEN +8.1% (heygotrade 10-28 close 363.21 +3.43%; gurufocus +3.4% same evening). Unresolved, left at their verified 10-27 close: CDNS 343.08, CRDO 167.43, AVAV 126.73, CEG 258.98 (heygotrade 10-27 closes match the board to the cent; no readable 10-28 close). SPY 772.31 10-28 (marketchameleon dated close; SSGA official 10-27 769.66 added to risk_series with ycharts ust10 4.99 10-27; ust10 10-28 skipped - named sources not yet updated, fool.com wrap printed 5.02 at close for reference). HISTORY 10-28 row mv updated in place for the new ETN/GEV closes. || PREVIOUS ENTRY: Oct 29, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: 48 of 63 set to the Wed 2026-10-28 close (fool.com dated quote pages; stockanalysis/Google Finance/ycharts caches frozen pre-close for a third night). 15 unresolved stay at their prior close: holdings CDNS CRDO AVAV GEV ETN CEG (10-27), watch ARM MPWR COHR SPCX LHX PWR GE TSEM CIEN (10-26). QQQ 725.61 (10-28); SPY, spyHigh and risk_series spy/ust10 left unchanged - no clean close readable. HISTORY row 10-28 added. 6%-movers verified: ORCL 144.54 +10.73% d/d, VRT 242.94 +16.49% d/d, MU 983.23, SNDK 1404.77, STX 697.97 (247wallst sidebar matches to the cent); SNPS FN BE STRL on dated fool closes + headline corroboration. || PREVIOUS ENTRY: Oct 29, 2026 - GOOGL TEST APPROVED (Salee): 19 Nov $18,524 tranche moved to a 10 Dec DECIDE - buy only if no further share sale AND a credible path back to positive free cash flow; fail = budget cut to cost spent, no sale. || PREVIOUS ENTRY: Oct 29, 2026 04:45 Bangkok - RESULTS SCORED: MSFT PASS (BUY 9 sh tonight, limit 531.01, cap 536.32); STRL FAIL (signed backlog 4.14bn &lt; 4.33bn; budget back to pool; half 2 cancelled); GEV thesis intact (Power orders +178%, Electrification -9% on a tough comparison); VRT partial disclosure; GOOGL Q3 cloud doubled but FCF -9.1bn + June 84.75bn equity raise - 19 Nov tranche pending Salee. Fed held 3.75-4.00% (10-2, Cook and Hammack for a hike). SGOV 4 Nov sale no longer needed. || PREVIOUS ENTRY: Oct 28, 2026 - SGOV SLICE 1 BOOKED: SELL 100 at 100.6901 = 10,047.46 net (POEMS 1187938, 22:29 Bangkok). Cash 29,714.36; SGOV 694 sh parked (cost 69,917.06). || PREVIOUS ENTRY: Oct 28, 2026 13:16 Bangkok - PRICES OF THE 36 HOLDINGS SET TO THE TUE 2026-10-27 CLOSE FROM SALEE'S POEMS POSITIONS SCREEN (US market closed; POEMS "Current Price" column; SGOV mark 100.68). Reason: every web source reachable from the sandbox served pre-close cached pages for Oct 27 through both scheduled runs (00:30 and 03:30 UTC) and manual checks at 03:30-04:50 UTC, so 0 of 63 could be written by the job. The 27 watch names (no position) stay at the 26 Oct close until the next successful run. Moves of 6%+ vs 26 Oct: CDNS +6.5%, ALAB +10.5%, CRDO +10.8%, RKLB +8.3% - consistent with the reported 27 Oct session (AMD +5.5%, AVGO +4%, MU +2.8%, chips rally). Positions and cost on the same screen reconcile to the board to the cent on all 36 lines (641,827.76 NASD + 247,167.89 NYSE incl. SGOV = 888,995.64). pe/ps/fpe/peg/pfcf rescaled with price per the 26 Oct rule. || PREVIOUS ENTRY: Oct 28, 2026 (runs 00:30 + 03:30 UTC) - DAILY PRICE REFRESH: BOTH overnight passes could not resolve the Tue 2026-10-27 close for any ticker. 03:30 pass sampled 14 stockanalysis.com quote/history pages: every capture predated the 4:00 PM close (freshest stamps 10:05-11:25 AM EDT Oct 27; some caches as old as May 2025), and Google Finance (Sep 24/25 caches), marketscreener (Sep 4) and ycharts (Oct 26 18:04 EDT) were equally stale. Per the leave-unchanged rule nothing was written: all 63 prices, mcaps, P/E block, SPY/QQQ and pxd stay at the Mon 2026-10-26 close (CGNX still 2026-10-23); no HISTORY row; risk_series ust10/spy 10-27 skipped (sources unreadable; ust10 2026-10-26 = 5.00 was already added by the 00:30 pass). Oct-26 baseline cross-checked against 9 history tables - all matched. Every number checked came from a tool call this session; the next scheduled pass retries.</t>
+          <t>Oct 30, 2026 21:45 Bangkok - CAT BOOKED: 7 sh at 633.5642 = 4,444.44 (rung 2 of 3; Power Generation test passed). Position 13 sh, cost 9,332.99; cash 20,530.86. October MONTHLY and investedEver updated with the fill. || PREVIOUS ENTRY: Oct 30, 2026 11:10 Bangkok - POEMS POSITIONS RECONCILED (screen 10:56 SGT, after the 29 Oct close): 36 lines + SGOV match to the cent; market value 874,941.02 ties. Nine NYSE marks set from POEMS (APH 82.08, ANET 184.22, CAT 647.39, ETN 393.72, TSM 431.81, VRT 245.92, V 410.54, VST 140.95; SGOV 100.71) - all within 0.2% of the job's closes; ratios rescaled. No fill tonight yet: CAT 7 sh LIMIT 647.39 (cap 653.86) is the only order. || PREVIOUS ENTRY: Oct 30, 2026 08:40 Bangkok - AMZN Q3 read recorded (AWS +39%, backlog $578bn, TTM FCF -$42.4bn, no order - over budget); CAT order set: 7 sh Day LIMIT 647.22, cap 653.69. || PREVIOUS ENTRY: Oct 30, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: all 63 prices set to the Thu 2026-10-29 close. Primary source this run: marketbeat.com dated daily-price tables / closing-price headers (pages updated 10/29, 'Closing price 4:00 PM Eastern' stamps), every ticker's prior close cross-checked against the stored board value; stockanalysis.com and Google Finance caches still frozen pre-close (5th night); GEV from the fool.com quote page previous-close field (887.85; method validated to the cent on GOOGL and MSFT this run). Big earnings-reaction day: 6%-movers verified + allowed: GOOGL 283.82 -12.64% (Q3 miss/FCF, fool prev-close field exact + news), FTNT 139.10 -20.09% (service-revenue forecast cut; 247wallst sidebar exact), MRVL 218.34 -13.24% (Lumentum deal talks; fool widget -13.24% exact), CAT 647.22 -9.49% (sales outlook; 247wallst sidebar 647.39), LHX 279.12 +7.10% (Q3 beat + raised FY guide; investing.com 278.65 +6.92%), AVAV 134.88 +7.09% (gurufocus +7.1%). SPY 769.36 and QQQ 715.34 (10-29, marketbeat closing headers; prev closes match board); spyHigh unchanged 779.09. risk_series spy 10-29 added; ust10 10-29 skipped (ycharts H15 only through 10-27; yahoo close bar printed 4.99 for reference). HISTORY 10-29 row added (first row including the 29 Oct MSFT buy, 126 sh). Note: TSEM 187.92 written from a dated 10/29 marketbeat header whose implied 10/28 prev close (193.52) could not be cross-checked - flagged for the next run. Every number from a tool call this session. || PREVIOUS ENTRY: Oct 29, 2026 23:00 Bangkok - GOOGL 10 Dec test (1) CLARIFIED: Q3 ATM share sales of $12.4bn were draws under the $40bn ATM announced in the June $84.75bn raise, so they do not fail the test; a new or upsized programme would. No order, budget or price changed. || PREVIOUS ENTRY: Oct 29, 2026 22:30 Bangkok - MSFT BOOKED 9 sh at 525.4031 = 4,738.75; cash 24,975.30. FULL POEMS RECONCILIATION: 36 lines + SGOV match to the cent; cash corrected by 0.10 (CRWD 19 Oct fee true-up); SGOV sale trued up to 10,047.25 (realised -27.25); October MONTHLY rebuilt (6 buys + 1 sale had been missing); October dividends 251.31 itemised. Prices: 54 names at the 28 Oct close, 9 at 27 Oct - the 29 Oct close is written by the next morning run. || PREVIOUS ENTRY: Oct 29, 2026 (03:30 UTC job) - DAILY PRICE REFRESH, 2nd pass: 11 more of the 15 stragglers resolved. Wed 2026-10-28 close written for ETN 392.88, GEV 878.03, PWR 606.89, COHR 239.59, SPCX 145.23, CIEN 363.21 (54 of 63 now at 10-28); verified Tue 10-27 close written for ARM 226.60, GE 297.66, MPWR 1211.89, LHX 259.40, TSEM 189.08 (marketbeat prev-close fields / heygotrade dated closes; every prev-close cross-checked against the stored prior close to the cent). Sources: 247wallst Oct-28 article sidebars validated to the cent on MSFT/ORCL/NVDA/MU/GOOGL/VRT; heygotrade dated close pages; stockanalysis/Google Finance/tipranks/marketscreener caches still frozen pre-close (4th night). 6%-movers vs last build, verified + allowed: PWR +7.6% (sidebar + 247wallst company page, prev 578.8x both), COHR +8.2% (sidebar; prev 235.79 = heygotrade 10-27 close exact), CIEN +8.1% (heygotrade 10-28 close 363.21 +3.43%; gurufocus +3.4% same evening). Unresolved, left at their verified 10-27 close: CDNS 343.08, CRDO 167.43, AVAV 126.73, CEG 258.98 (heygotrade 10-27 closes match the board to the cent; no readable 10-28 close). SPY 772.31 10-28 (marketchameleon dated close; SSGA official 10-27 769.66 added to risk_series with ycharts ust10 4.99 10-27; ust10 10-28 skipped - named sources not yet updated, fool.com wrap printed 5.02 at close for reference). HISTORY 10-28 row mv updated in place for the new ETN/GEV closes. || PREVIOUS ENTRY: Oct 29, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: 48 of 63 set to the Wed 2026-10-28 close (fool.com dated quote pages; stockanalysis/Google Finance/ycharts caches frozen pre-close for a third night). 15 unresolved stay at their prior close: holdings CDNS CRDO AVAV GEV ETN CEG (10-27), watch ARM MPWR COHR SPCX LHX PWR GE TSEM CIEN (10-26). QQQ 725.61 (10-28); SPY, spyHigh and risk_series spy/ust10 left unchanged - no clean close readable. HISTORY row 10-28 added. 6%-movers verified: ORCL 144.54 +10.73% d/d, VRT 242.94 +16.49% d/d, MU 983.23, SNDK 1404.77, STX 697.97 (247wallst sidebar matches to the cent); SNPS FN BE STRL on dated fool closes + headline corroboration. || PREVIOUS ENTRY: Oct 29, 2026 - GOOGL TEST APPROVED (Salee): 19 Nov $18,524 tranche moved to a 10 Dec DECIDE - buy only if no further share sale AND a credible path back to positive free cash flow; fail = budget cut to cost spent, no sale. || PREVIOUS ENTRY: Oct 29, 2026 04:45 Bangkok - RESULTS SCORED: MSFT PASS (BUY 9 sh tonight, limit 531.01, cap 536.32); STRL FAIL (signed backlog 4.14bn &lt; 4.33bn; budget back to pool; half 2 cancelled); GEV thesis intact (Power orders +178%, Electrification -9% on a tough comparison); VRT partial disclosure; GOOGL Q3 cloud doubled but FCF -9.1bn + June 84.75bn equity raise - 19 Nov tranche pending Salee. Fed held 3.75-4.00% (10-2, Cook and Hammack for a hike). SGOV 4 Nov sale no longer needed. || PREVIOUS ENTRY: Oct 28, 2026 - SGOV SLICE 1 BOOKED: SELL 100 at 100.6901 = 10,047.46 net (POEMS 1187938, 22:29 Bangkok). Cash 29,714.36; SGOV 694 sh parked (cost 69,917.06). || PREVIOUS ENTRY: Oct 28, 2026 13:16 Bangkok - PRICES OF THE 36 HOLDINGS SET TO THE TUE 2026-10-27 CLOSE FROM SALEE'S POEMS POSITIONS SCREEN (US market closed; POEMS "Current Price" column; SGOV mark 100.68). Reason: every web source reachable from the sandbox served pre-close cached pages for Oct 27 through both scheduled runs (00:30 and 03:30 UTC) and manual checks at 03:30-04:50 UTC, so 0 of 63 could be written by the job. The 27 watch names (no position) stay at the 26 Oct close until the next successful run. Moves of 6%+ vs 26 Oct: CDNS +6.5%, ALAB +10.5%, CRDO +10.8%, RKLB +8.3% - consistent with the reported 27 Oct session (AMD +5.5%, AVGO +4%, MU +2.8%, chips rally). Positions and cost on the same screen reconcile to the board to the cent on all 36 lines (641,827.76 NASD + 247,167.89 NYSE incl. SGOV = 888,995.64). pe/ps/fpe/peg/pfcf rescaled with price per the 26 Oct rule. || PREVIOUS ENTRY: Oct 28, 2026 (runs 00:30 + 03:30 UTC) - DAILY PRICE REFRESH: BOTH overnight passes could not resolve the Tue 2026-10-27 close for any ticker. 03:30 pass sampled 14 stockanalysis.com quote/history pages: every capture predated the 4:00 PM close (freshest stamps 10:05-11:25 AM EDT Oct 27; some caches as old as May 2025), and Google Finance (Sep 24/25 caches), marketscreener (Sep 4) and ycharts (Oct 26 18:04 EDT) were equally stale. Per the leave-unchanged rule nothing was written: all 63 prices, mcaps, P/E block, SPY/QQQ and pxd stay at the Mon 2026-10-26 close (CGNX still 2026-10-23); no HISTORY row; risk_series ust10/spy 10-27 skipped (sources unreadable; ust10 2026-10-26 = 5.00 was already added by the 00:30 pass). Oct-26 baseline cross-checked against 9 history tables - all matched. Every number checked came from a tool call this session; the next scheduled pass retries.</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>723713.41</v>
+        <v>728157.85</v>
       </c>
     </row>
     <row r="5">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>805048.28</v>
+        <v>809580.01</v>
       </c>
     </row>
     <row r="6">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>81334.87</v>
+        <v>81422.16</v>
       </c>
     </row>
     <row r="7">
@@ -517,7 +517,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>+11.24%</t>
+          <t>+11.18%</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>24975.3</v>
+        <v>20530.86</v>
       </c>
     </row>
     <row r="10">
@@ -549,7 +549,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Oct 29, 2026 22:16 Bangkok - POEMS Cash Balance (Live) 29,714.05 after the SGOV sale (10,047.25), before the MSFT buy; less MSFT 9 sh at 525.4031 = 4,738.75 (est. commission) = 24,975.30. Board now matches POEMS to the cent (the +0.10 carried since 19 Oct is removed). || PREVIOUS: Oct 28, 2026 - after SGOV sale 100 sh at 100.6901 = 10,047.46 net of est. commission: 19,666.90 + 10,047.46 = 29,714.36 (proceeds settle 29 Oct). POEMS Live Cash Balance read 22:30 Bangkok BEFORE the sale: 19,666.80 (board 19,666.90 - 10 cents, carried from 26 Oct). SGOV 694 sh parked. || PREVIOUS: Oct 26, 2026 - after CRDO buy 34 sh at 148.76 = 5,068.66 incl. est. commission: 24,735.56 - 5,068.66 = 19,666.90. POEMS Live Cash Balance read 21:15 Bangkok before the order: 24,735.46 (10 cents below the board's 24,735.56 - to itemise at the next statement). SGOV 794 sh parked. || PREVIOUS: Oct 22, 2026 - after META buy 18 sh at 658.5807 = 11,879.82 incl. est. commission: 36,615.38 - 11,879.82 = 24,735.56. SGOV 794 sh parked. || PREVIOUS: Oct 19, 2026 - after tonight's two fills: CRWD sale +4,573.49 (est. fees) and NVDA buy -6,921.92 (est. commission): 38,963.81 + 4,573.49 - 6,921.92 = 36,615.38. CRWD proceeds settle T+1. SGOV 794 sh still parked. To be read against the POEMS Live Cash Balance. || PREVIOUS: Oct 16, 2026 - POEMS Live Cash Balance 06:45 am Bangkok: USD 55,058.84, shown BEFORE settlement of the 15 Oct buys. Board cash = 55,058.84 less TSM 9,621.29 and ASML 6,473.74 = 38,963.81 after settlement. Versus the derived 55,050.83, POEMS is +8.01 higher with no trades in between - a small credit (interest or dividend) to itemise from the October statement with the earlier +146.84 and +96.46. Positions reconciled the same morning: 37 stock lines + SGOV, cost 777,052.88, match POEMS to the cent, and the POEMS cost on TSM (64,477.71) and ASML (22,867.80) confirms the two commission estimates exactly. || PREVIOUS: Oct 15, 2026 - after tonight's two fills (TSM 23 sh 9,621.29, ASML 4 sh 6,473.74, both incl. estimated commission) totalling 16,095.03: 55,050.83 - 16,095.03 = 38,955.80. SGOV 79,991.56 still parked, so total liquid = 118,947.36. To be read against the POEMS Live Cash Balance after T+1 settlement. || PREVIOUS: Oct 13, 2026 - SGOV PARK FILLED: 794 sh at 100.5299 (POEMS, Done 11:04:13 pm Bangkok) = gross 79,820.74 + est. commission 170.82 = 79,991.56. Free cash 135,042.39 - 79,991.56 = 55,050.83. SGOV held as a cash-equivalent (see parked), so total liquid = 135,042.39. To be read against the POEMS Live Cash Balance after T+1 settlement. || PREVIOUS: Oct 13, 2026 - after the 12 Oct fills (APH, CRDO, V) totalling 12,973.99 incl. estimated commission: 148,016.38 - 12,973.99 = 135,042.39. To be read against the POEMS Live Cash Balance after settlement. || PREVIOUS: Oct 10, 2026 - POEMS Live Cash Balance 07:53 am Bangkok: USD 170,344.36, shown BEFORE settlement of the 9 Oct buys. Board cash = 170,344.36 less MRVL 12,712.45 and AMAT 9,615.53 = 148,016.38 after settlement. Versus the 6 Oct balance of 170,247.90, POEMS is +96.46 higher with no trades in between - a further early-October credit (most likely dividends), to itemise from the October statement together with the earlier +146.84. Positions reconciled the same morning: 37 lines, cost 667,992.30, match POEMS to the cent. || PREVIOUS: Oct 6, 2026 - POEMS Live Cash Balance 170,247.90. RECONCILED 7 Oct: POEMS statement cash at 30 Sep = 168,539.69; less MU buy 1 Oct 14,703.40, plus ORCL 10,851.50 and CRWD 5,413.27 sale proceeds = 170,101.06; the remaining +146.84 is early-October credits (most likely dividends) to itemise from the October statement. (The earlier +172.61 figure came from a board-derived cash that was 25.77 too low.) || PREVIOUS: Oct 6, 2026 - read off the POEMS Live Cash Balance screen (09:23 am, before settlement of the 5 Oct sales): USD 170,247.90. Derived from the board: 153,810.52 + 10,851.50 (ORCL) + 5,413.27 (CRWD) = 170,075.29; POEMS is +172.61 higher - most likely dividends/interest credited since 2 Oct, to be itemised. || PREVIOUS: Oct 2, 2026 (153862.15 less 51.63 of commission under-booked on the five orders of 28 Sep and 1 Oct, found when the POEMS positions screen of 2 Oct was reconciled. Positions now match POEMS to the cent on all 38 lines. Cash itself is derived, not yet read off a POEMS cash screen)</t>
+          <t>Oct 30, 2026 21:35 Bangkok - after CAT buy 7 sh at 633.5642 = 4,444.44 (est. commission): 24,975.30 - 4,444.44 = 20,530.86. To be read against the POEMS Live Cash Balance (the app's SGD buying power is not comparable). || PREVIOUS: Oct 29, 2026 22:16 Bangkok - POEMS Cash Balance (Live) 29,714.05 after the SGOV sale (10,047.25), before the MSFT buy; less MSFT 9 sh at 525.4031 = 4,738.75 (est. commission) = 24,975.30. Board now matches POEMS to the cent (the +0.10 carried since 19 Oct is removed). || PREVIOUS: Oct 28, 2026 - after SGOV sale 100 sh at 100.6901 = 10,047.46 net of est. commission: 19,666.90 + 10,047.46 = 29,714.36 (proceeds settle 29 Oct). POEMS Live Cash Balance read 22:30 Bangkok BEFORE the sale: 19,666.80 (board 19,666.90 - 10 cents, carried from 26 Oct). SGOV 694 sh parked. || PREVIOUS: Oct 26, 2026 - after CRDO buy 34 sh at 148.76 = 5,068.66 incl. est. commission: 24,735.56 - 5,068.66 = 19,666.90. POEMS Live Cash Balance read 21:15 Bangkok before the order: 24,735.46 (10 cents below the board's 24,735.56 - to itemise at the next statement). SGOV 794 sh parked. || PREVIOUS: Oct 22, 2026 - after META buy 18 sh at 658.5807 = 11,879.82 incl. est. commission: 36,615.38 - 11,879.82 = 24,735.56. SGOV 794 sh parked. || PREVIOUS: Oct 19, 2026 - after tonight's two fills: CRWD sale +4,573.49 (est. fees) and NVDA buy -6,921.92 (est. commission): 38,963.81 + 4,573.49 - 6,921.92 = 36,615.38. CRWD proceeds settle T+1. SGOV 794 sh still parked. To be read against the POEMS Live Cash Balance. || PREVIOUS: Oct 16, 2026 - POEMS Live Cash Balance 06:45 am Bangkok: USD 55,058.84, shown BEFORE settlement of the 15 Oct buys. Board cash = 55,058.84 less TSM 9,621.29 and ASML 6,473.74 = 38,963.81 after settlement. Versus the derived 55,050.83, POEMS is +8.01 higher with no trades in between - a small credit (interest or dividend) to itemise from the October statement with the earlier +146.84 and +96.46. Positions reconciled the same morning: 37 stock lines + SGOV, cost 777,052.88, match POEMS to the cent, and the POEMS cost on TSM (64,477.71) and ASML (22,867.80) confirms the two commission estimates exactly. || PREVIOUS: Oct 15, 2026 - after tonight's two fills (TSM 23 sh 9,621.29, ASML 4 sh 6,473.74, both incl. estimated commission) totalling 16,095.03: 55,050.83 - 16,095.03 = 38,955.80. SGOV 79,991.56 still parked, so total liquid = 118,947.36. To be read against the POEMS Live Cash Balance after T+1 settlement. || PREVIOUS: Oct 13, 2026 - SGOV PARK FILLED: 794 sh at 100.5299 (POEMS, Done 11:04:13 pm Bangkok) = gross 79,820.74 + est. commission 170.82 = 79,991.56. Free cash 135,042.39 - 79,991.56 = 55,050.83. SGOV held as a cash-equivalent (see parked), so total liquid = 135,042.39. To be read against the POEMS Live Cash Balance after T+1 settlement. || PREVIOUS: Oct 13, 2026 - after the 12 Oct fills (APH, CRDO, V) totalling 12,973.99 incl. estimated commission: 148,016.38 - 12,973.99 = 135,042.39. To be read against the POEMS Live Cash Balance after settlement. || PREVIOUS: Oct 10, 2026 - POEMS Live Cash Balance 07:53 am Bangkok: USD 170,344.36, shown BEFORE settlement of the 9 Oct buys. Board cash = 170,344.36 less MRVL 12,712.45 and AMAT 9,615.53 = 148,016.38 after settlement. Versus the 6 Oct balance of 170,247.90, POEMS is +96.46 higher with no trades in between - a further early-October credit (most likely dividends), to itemise from the October statement together with the earlier +146.84. Positions reconciled the same morning: 37 lines, cost 667,992.30, match POEMS to the cent. || PREVIOUS: Oct 6, 2026 - POEMS Live Cash Balance 170,247.90. RECONCILED 7 Oct: POEMS statement cash at 30 Sep = 168,539.69; less MU buy 1 Oct 14,703.40, plus ORCL 10,851.50 and CRWD 5,413.27 sale proceeds = 170,101.06; the remaining +146.84 is early-October credits (most likely dividends) to itemise from the October statement. (The earlier +172.61 figure came from a board-derived cash that was 25.77 too low.) || PREVIOUS: Oct 6, 2026 - read off the POEMS Live Cash Balance screen (09:23 am, before settlement of the 5 Oct sales): USD 170,247.90. Derived from the board: 153,810.52 + 10,851.50 (ORCL) + 5,413.27 (CRWD) = 170,075.29; POEMS is +172.61 higher - most likely dividends/interest credited since 2 Oct, to be itemised. || PREVIOUS: Oct 2, 2026 (153862.15 less 51.63 of commission under-booked on the five orders of 28 Sep and 1 Oct, found when the POEMS positions screen of 2 Oct was reconciled. Positions now match POEMS to the cent on all 38 lines. Cash itself is derived, not yet read off a POEMS cash screen)</t>
         </is>
       </c>
     </row>
@@ -2311,34 +2311,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>4888.55</v>
+        <v>9332.99</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>814.7583333333333</v>
+        <v>717.9223076923076</v>
       </c>
       <c r="G37" s="3" t="n">
         <v>647.39</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>3884.34</v>
+        <v>8416.07</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-1004.21</v>
+        <v>-916.9200000000001</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>-0.2054208303075554</v>
+        <v>-0.09824504258549512</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>33.65</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>164499.7075</v>
+        <v>314055.1135</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>130708.041</v>
+        <v>283200.7555</v>
       </c>
     </row>
     <row r="38">
@@ -2348,16 +2348,16 @@
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>723713.41</v>
+        <v>728157.85</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>805048.2814999999</v>
+        <v>809580.0115</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>81334.87149999989</v>
+        <v>81422.16150000005</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>0.112385469684747</v>
+        <v>0.1118193829813138</v>
       </c>
     </row>
   </sheetData>
@@ -7885,7 +7885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H251"/>
+  <dimension ref="A1:H252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -16437,6 +16437,40 @@
       <c r="H251" t="inlineStr">
         <is>
           <t>MSFT final rung - Q1 FY27 test PASSED (Azure +48%, quarter capex $45.2bn under its own ~$50bn guide, capex plan maintained). Day LIMIT 531.01 (28 Oct close) placed with the stock at ~$525 after the post-results pop faded in a tech sell-off; Done 22:15:19 Bangkok at 525.4031. Gross 4,728.63 + est. commission 10.12 = 4,738.75. Position 126 sh, cost 57,617.71 of 58,000 (room 382.29) - budget effectively full.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Oct 30, 2026</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>7</v>
+      </c>
+      <c r="E252" s="3" t="n">
+        <v>633.5642</v>
+      </c>
+      <c r="F252" s="3" t="n">
+        <v>4444.44</v>
+      </c>
+      <c r="G252" t="b">
+        <v>1</v>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>CATERPILLAR RUNG 2 OF 3 - Q3 test PASSED 29 Oct (Power Generation sales $3.42bn, +30%). Stock fell 9.5% on 29 Oct (outlook not raised) and a further ~2% on 30 Oct; Day LIMIT lowered to 636.00 with the price at 633.81 (reference close 647.39, cap 653.86). Done 21:35 Bangkok at 633.5642. Gross 4,434.95 + est. commission 9.49 (0.214%) = 4,444.44. Position 13 sh, cost 9,332.99 of 15,000; rung 3 ($5,000) on 11 Nov.</t>
         </is>
       </c>
     </row>
@@ -16882,10 +16916,10 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>94709.55</v>
+        <v>99153.99000000001</v>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>20838.16</v>

</xml_diff>

<commit_message>
31 Oct: all 63 prices at the Fri 30 Oct close - 36 holdings from POEMS (cost 798,074.91 / MV 843,570.71 tie), 27 watch names verified; SPY/QQQ; HISTORY 10-30; workbook rebuilt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJZYTemDPd8XNBcdUBVnWw
</commit_message>
<xml_diff>
--- a/src/Pillar4_US_Portfolio_Workbook.xlsx
+++ b/src/Pillar4_US_Portfolio_Workbook.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oct 30, 2026 21:45 Bangkok - CAT BOOKED: 7 sh at 633.5642 = 4,444.44 (rung 2 of 3; Power Generation test passed). Position 13 sh, cost 9,332.99; cash 20,530.86. October MONTHLY and investedEver updated with the fill. || PREVIOUS ENTRY: Oct 30, 2026 11:10 Bangkok - POEMS POSITIONS RECONCILED (screen 10:56 SGT, after the 29 Oct close): 36 lines + SGOV match to the cent; market value 874,941.02 ties. Nine NYSE marks set from POEMS (APH 82.08, ANET 184.22, CAT 647.39, ETN 393.72, TSM 431.81, VRT 245.92, V 410.54, VST 140.95; SGOV 100.71) - all within 0.2% of the job's closes; ratios rescaled. No fill tonight yet: CAT 7 sh LIMIT 647.39 (cap 653.86) is the only order. || PREVIOUS ENTRY: Oct 30, 2026 08:40 Bangkok - AMZN Q3 read recorded (AWS +39%, backlog $578bn, TTM FCF -$42.4bn, no order - over budget); CAT order set: 7 sh Day LIMIT 647.22, cap 653.69. || PREVIOUS ENTRY: Oct 30, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: all 63 prices set to the Thu 2026-10-29 close. Primary source this run: marketbeat.com dated daily-price tables / closing-price headers (pages updated 10/29, 'Closing price 4:00 PM Eastern' stamps), every ticker's prior close cross-checked against the stored board value; stockanalysis.com and Google Finance caches still frozen pre-close (5th night); GEV from the fool.com quote page previous-close field (887.85; method validated to the cent on GOOGL and MSFT this run). Big earnings-reaction day: 6%-movers verified + allowed: GOOGL 283.82 -12.64% (Q3 miss/FCF, fool prev-close field exact + news), FTNT 139.10 -20.09% (service-revenue forecast cut; 247wallst sidebar exact), MRVL 218.34 -13.24% (Lumentum deal talks; fool widget -13.24% exact), CAT 647.22 -9.49% (sales outlook; 247wallst sidebar 647.39), LHX 279.12 +7.10% (Q3 beat + raised FY guide; investing.com 278.65 +6.92%), AVAV 134.88 +7.09% (gurufocus +7.1%). SPY 769.36 and QQQ 715.34 (10-29, marketbeat closing headers; prev closes match board); spyHigh unchanged 779.09. risk_series spy 10-29 added; ust10 10-29 skipped (ycharts H15 only through 10-27; yahoo close bar printed 4.99 for reference). HISTORY 10-29 row added (first row including the 29 Oct MSFT buy, 126 sh). Note: TSEM 187.92 written from a dated 10/29 marketbeat header whose implied 10/28 prev close (193.52) could not be cross-checked - flagged for the next run. Every number from a tool call this session. || PREVIOUS ENTRY: Oct 29, 2026 23:00 Bangkok - GOOGL 10 Dec test (1) CLARIFIED: Q3 ATM share sales of $12.4bn were draws under the $40bn ATM announced in the June $84.75bn raise, so they do not fail the test; a new or upsized programme would. No order, budget or price changed. || PREVIOUS ENTRY: Oct 29, 2026 22:30 Bangkok - MSFT BOOKED 9 sh at 525.4031 = 4,738.75; cash 24,975.30. FULL POEMS RECONCILIATION: 36 lines + SGOV match to the cent; cash corrected by 0.10 (CRWD 19 Oct fee true-up); SGOV sale trued up to 10,047.25 (realised -27.25); October MONTHLY rebuilt (6 buys + 1 sale had been missing); October dividends 251.31 itemised. Prices: 54 names at the 28 Oct close, 9 at 27 Oct - the 29 Oct close is written by the next morning run. || PREVIOUS ENTRY: Oct 29, 2026 (03:30 UTC job) - DAILY PRICE REFRESH, 2nd pass: 11 more of the 15 stragglers resolved. Wed 2026-10-28 close written for ETN 392.88, GEV 878.03, PWR 606.89, COHR 239.59, SPCX 145.23, CIEN 363.21 (54 of 63 now at 10-28); verified Tue 10-27 close written for ARM 226.60, GE 297.66, MPWR 1211.89, LHX 259.40, TSEM 189.08 (marketbeat prev-close fields / heygotrade dated closes; every prev-close cross-checked against the stored prior close to the cent). Sources: 247wallst Oct-28 article sidebars validated to the cent on MSFT/ORCL/NVDA/MU/GOOGL/VRT; heygotrade dated close pages; stockanalysis/Google Finance/tipranks/marketscreener caches still frozen pre-close (4th night). 6%-movers vs last build, verified + allowed: PWR +7.6% (sidebar + 247wallst company page, prev 578.8x both), COHR +8.2% (sidebar; prev 235.79 = heygotrade 10-27 close exact), CIEN +8.1% (heygotrade 10-28 close 363.21 +3.43%; gurufocus +3.4% same evening). Unresolved, left at their verified 10-27 close: CDNS 343.08, CRDO 167.43, AVAV 126.73, CEG 258.98 (heygotrade 10-27 closes match the board to the cent; no readable 10-28 close). SPY 772.31 10-28 (marketchameleon dated close; SSGA official 10-27 769.66 added to risk_series with ycharts ust10 4.99 10-27; ust10 10-28 skipped - named sources not yet updated, fool.com wrap printed 5.02 at close for reference). HISTORY 10-28 row mv updated in place for the new ETN/GEV closes. || PREVIOUS ENTRY: Oct 29, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: 48 of 63 set to the Wed 2026-10-28 close (fool.com dated quote pages; stockanalysis/Google Finance/ycharts caches frozen pre-close for a third night). 15 unresolved stay at their prior close: holdings CDNS CRDO AVAV GEV ETN CEG (10-27), watch ARM MPWR COHR SPCX LHX PWR GE TSEM CIEN (10-26). QQQ 725.61 (10-28); SPY, spyHigh and risk_series spy/ust10 left unchanged - no clean close readable. HISTORY row 10-28 added. 6%-movers verified: ORCL 144.54 +10.73% d/d, VRT 242.94 +16.49% d/d, MU 983.23, SNDK 1404.77, STX 697.97 (247wallst sidebar matches to the cent); SNPS FN BE STRL on dated fool closes + headline corroboration. || PREVIOUS ENTRY: Oct 29, 2026 - GOOGL TEST APPROVED (Salee): 19 Nov $18,524 tranche moved to a 10 Dec DECIDE - buy only if no further share sale AND a credible path back to positive free cash flow; fail = budget cut to cost spent, no sale. || PREVIOUS ENTRY: Oct 29, 2026 04:45 Bangkok - RESULTS SCORED: MSFT PASS (BUY 9 sh tonight, limit 531.01, cap 536.32); STRL FAIL (signed backlog 4.14bn &lt; 4.33bn; budget back to pool; half 2 cancelled); GEV thesis intact (Power orders +178%, Electrification -9% on a tough comparison); VRT partial disclosure; GOOGL Q3 cloud doubled but FCF -9.1bn + June 84.75bn equity raise - 19 Nov tranche pending Salee. Fed held 3.75-4.00% (10-2, Cook and Hammack for a hike). SGOV 4 Nov sale no longer needed. || PREVIOUS ENTRY: Oct 28, 2026 - SGOV SLICE 1 BOOKED: SELL 100 at 100.6901 = 10,047.46 net (POEMS 1187938, 22:29 Bangkok). Cash 29,714.36; SGOV 694 sh parked (cost 69,917.06). || PREVIOUS ENTRY: Oct 28, 2026 13:16 Bangkok - PRICES OF THE 36 HOLDINGS SET TO THE TUE 2026-10-27 CLOSE FROM SALEE'S POEMS POSITIONS SCREEN (US market closed; POEMS "Current Price" column; SGOV mark 100.68). Reason: every web source reachable from the sandbox served pre-close cached pages for Oct 27 through both scheduled runs (00:30 and 03:30 UTC) and manual checks at 03:30-04:50 UTC, so 0 of 63 could be written by the job. The 27 watch names (no position) stay at the 26 Oct close until the next successful run. Moves of 6%+ vs 26 Oct: CDNS +6.5%, ALAB +10.5%, CRDO +10.8%, RKLB +8.3% - consistent with the reported 27 Oct session (AMD +5.5%, AVGO +4%, MU +2.8%, chips rally). Positions and cost on the same screen reconcile to the board to the cent on all 36 lines (641,827.76 NASD + 247,167.89 NYSE incl. SGOV = 888,995.64). pe/ps/fpe/peg/pfcf rescaled with price per the 26 Oct rule. || PREVIOUS ENTRY: Oct 28, 2026 (runs 00:30 + 03:30 UTC) - DAILY PRICE REFRESH: BOTH overnight passes could not resolve the Tue 2026-10-27 close for any ticker. 03:30 pass sampled 14 stockanalysis.com quote/history pages: every capture predated the 4:00 PM close (freshest stamps 10:05-11:25 AM EDT Oct 27; some caches as old as May 2025), and Google Finance (Sep 24/25 caches), marketscreener (Sep 4) and ycharts (Oct 26 18:04 EDT) were equally stale. Per the leave-unchanged rule nothing was written: all 63 prices, mcaps, P/E block, SPY/QQQ and pxd stay at the Mon 2026-10-26 close (CGNX still 2026-10-23); no HISTORY row; risk_series ust10/spy 10-27 skipped (sources unreadable; ust10 2026-10-26 = 5.00 was already added by the 00:30 pass). Oct-26 baseline cross-checked against 9 history tables - all matched. Every number checked came from a tool call this session; the next scheduled pass retries.</t>
+          <t>Oct 31, 2026 09:50 Bangkok - ALL 63 PRICES AT THE FRI 30 OCT CLOSE (the 00:30 UTC price job did not run - scheduled jobs on claude-fable-5 are failing on the usage limit). 36 HOLDINGS from Salee's POEMS positions screen 09:36 SGT: all 36 lines + SGOV match quantity and cost to the cent incl. the 30 Oct CAT fill (cost 798,074.91; MV 843,570.71; CAT commission estimate 9.49 confirmed). 27 WATCH NAMES from marketbeat 10/30 4:00 PM closing headers / fool.com 'last close 2026-10-30' / massive.com / financialcontent, each cross-checked against the prior close or a second source. SPY 755.72 (-1.77%), QQQ 690.49 (-3.47%). Semiconductor sell-off day (Intel -29% on a weak Q4 guide; SOX about -7 to -9%): 6%+ moves verified - holdings AMD -10.9%, MRVL -10.0%, ALAB -10.9%, CRDO -8.7%, LITE -8.6%, ANET -8.3%, AMAT -7.5%, TER -7.4%, RKLB -7.4%, ASML -6.6%, AVAV -6.5%, PLTR -6.3%, LRCX -6.0%, ETN -6.0%; watch SNDK -13.5%, DDOG -11.5%, TSEM -11.4%, COHR -11.2%, APP -10.4%, ARM -10.0%, NET -9.5%, BE -8.6%, STX -8.0%, CIEN -8.0%, STRL -7.4%, HOOD -7.2%, SPCX -6.4%, ORCL -6.3%, FN -6.3%. Ratios rescaled with price. HISTORY 10-30 row added (stocks MV 773,664.08, unrealised +45,506.23 / +6.25%). Note: 8 NYSE watch closes of 29 Oct (COHR FN LHX ORCL NET PWR GE CIEN) were 3:59 PM prints, cents off the official close - superseded by today's verified closes. AMZN/CAT/LHX Q3 fundamentals still pending (earnings job failed). || PREVIOUS ENTRY: Oct 30, 2026 21:45 Bangkok - CAT BOOKED: 7 sh at 633.5642 = 4,444.44 (rung 2 of 3; Power Generation test passed). Position 13 sh, cost 9,332.99; cash 20,530.86. October MONTHLY and investedEver updated with the fill. || PREVIOUS ENTRY: Oct 30, 2026 11:10 Bangkok - POEMS POSITIONS RECONCILED (screen 10:56 SGT, after the 29 Oct close): 36 lines + SGOV match to the cent; market value 874,941.02 ties. Nine NYSE marks set from POEMS (APH 82.08, ANET 184.22, CAT 647.39, ETN 393.72, TSM 431.81, VRT 245.92, V 410.54, VST 140.95; SGOV 100.71) - all within 0.2% of the job's closes; ratios rescaled. No fill tonight yet: CAT 7 sh LIMIT 647.39 (cap 653.86) is the only order. || PREVIOUS ENTRY: Oct 30, 2026 08:40 Bangkok - AMZN Q3 read recorded (AWS +39%, backlog $578bn, TTM FCF -$42.4bn, no order - over budget); CAT order set: 7 sh Day LIMIT 647.22, cap 653.69. || PREVIOUS ENTRY: Oct 30, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: all 63 prices set to the Thu 2026-10-29 close. Primary source this run: marketbeat.com dated daily-price tables / closing-price headers (pages updated 10/29, 'Closing price 4:00 PM Eastern' stamps), every ticker's prior close cross-checked against the stored board value; stockanalysis.com and Google Finance caches still frozen pre-close (5th night); GEV from the fool.com quote page previous-close field (887.85; method validated to the cent on GOOGL and MSFT this run). Big earnings-reaction day: 6%-movers verified + allowed: GOOGL 283.82 -12.64% (Q3 miss/FCF, fool prev-close field exact + news), FTNT 139.10 -20.09% (service-revenue forecast cut; 247wallst sidebar exact), MRVL 218.34 -13.24% (Lumentum deal talks; fool widget -13.24% exact), CAT 647.22 -9.49% (sales outlook; 247wallst sidebar 647.39), LHX 279.12 +7.10% (Q3 beat + raised FY guide; investing.com 278.65 +6.92%), AVAV 134.88 +7.09% (gurufocus +7.1%). SPY 769.36 and QQQ 715.34 (10-29, marketbeat closing headers; prev closes match board); spyHigh unchanged 779.09. risk_series spy 10-29 added; ust10 10-29 skipped (ycharts H15 only through 10-27; yahoo close bar printed 4.99 for reference). HISTORY 10-29 row added (first row including the 29 Oct MSFT buy, 126 sh). Note: TSEM 187.92 written from a dated 10/29 marketbeat header whose implied 10/28 prev close (193.52) could not be cross-checked - flagged for the next run. Every number from a tool call this session. || PREVIOUS ENTRY: Oct 29, 2026 23:00 Bangkok - GOOGL 10 Dec test (1) CLARIFIED: Q3 ATM share sales of $12.4bn were draws under the $40bn ATM announced in the June $84.75bn raise, so they do not fail the test; a new or upsized programme would. No order, budget or price changed. || PREVIOUS ENTRY: Oct 29, 2026 22:30 Bangkok - MSFT BOOKED 9 sh at 525.4031 = 4,738.75; cash 24,975.30. FULL POEMS RECONCILIATION: 36 lines + SGOV match to the cent; cash corrected by 0.10 (CRWD 19 Oct fee true-up); SGOV sale trued up to 10,047.25 (realised -27.25); October MONTHLY rebuilt (6 buys + 1 sale had been missing); October dividends 251.31 itemised. Prices: 54 names at the 28 Oct close, 9 at 27 Oct - the 29 Oct close is written by the next morning run. || PREVIOUS ENTRY: Oct 29, 2026 (03:30 UTC job) - DAILY PRICE REFRESH, 2nd pass: 11 more of the 15 stragglers resolved. Wed 2026-10-28 close written for ETN 392.88, GEV 878.03, PWR 606.89, COHR 239.59, SPCX 145.23, CIEN 363.21 (54 of 63 now at 10-28); verified Tue 10-27 close written for ARM 226.60, GE 297.66, MPWR 1211.89, LHX 259.40, TSEM 189.08 (marketbeat prev-close fields / heygotrade dated closes; every prev-close cross-checked against the stored prior close to the cent). Sources: 247wallst Oct-28 article sidebars validated to the cent on MSFT/ORCL/NVDA/MU/GOOGL/VRT; heygotrade dated close pages; stockanalysis/Google Finance/tipranks/marketscreener caches still frozen pre-close (4th night). 6%-movers vs last build, verified + allowed: PWR +7.6% (sidebar + 247wallst company page, prev 578.8x both), COHR +8.2% (sidebar; prev 235.79 = heygotrade 10-27 close exact), CIEN +8.1% (heygotrade 10-28 close 363.21 +3.43%; gurufocus +3.4% same evening). Unresolved, left at their verified 10-27 close: CDNS 343.08, CRDO 167.43, AVAV 126.73, CEG 258.98 (heygotrade 10-27 closes match the board to the cent; no readable 10-28 close). SPY 772.31 10-28 (marketchameleon dated close; SSGA official 10-27 769.66 added to risk_series with ycharts ust10 4.99 10-27; ust10 10-28 skipped - named sources not yet updated, fool.com wrap printed 5.02 at close for reference). HISTORY 10-28 row mv updated in place for the new ETN/GEV closes. || PREVIOUS ENTRY: Oct 29, 2026 (00:30 UTC job) - DAILY PRICE REFRESH: 48 of 63 set to the Wed 2026-10-28 close (fool.com dated quote pages; stockanalysis/Google Finance/ycharts caches frozen pre-close for a third night). 15 unresolved stay at their prior close: holdings CDNS CRDO AVAV GEV ETN CEG (10-27), watch ARM MPWR COHR SPCX LHX PWR GE TSEM CIEN (10-26). QQQ 725.61 (10-28); SPY, spyHigh and risk_series spy/ust10 left unchanged - no clean close readable. HISTORY row 10-28 added. 6%-movers verified: ORCL 144.54 +10.73% d/d, VRT 242.94 +16.49% d/d, MU 983.23, SNDK 1404.77, STX 697.97 (247wallst sidebar matches to the cent); SNPS FN BE STRL on dated fool closes + headline corroboration. || PREVIOUS ENTRY: Oct 29, 2026 - GOOGL TEST APPROVED (Salee): 19 Nov $18,524 tranche moved to a 10 Dec DECIDE - buy only if no further share sale AND a credible path back to positive free cash flow; fail = budget cut to cost spent, no sale. || PREVIOUS ENTRY: Oct 29, 2026 04:45 Bangkok - RESULTS SCORED: MSFT PASS (BUY 9 sh tonight, limit 531.01, cap 536.32); STRL FAIL (signed backlog 4.14bn &lt; 4.33bn; budget back to pool; half 2 cancelled); GEV thesis intact (Power orders +178%, Electrification -9% on a tough comparison); VRT partial disclosure; GOOGL Q3 cloud doubled but FCF -9.1bn + June 84.75bn equity raise - 19 Nov tranche pending Salee. Fed held 3.75-4.00% (10-2, Cook and Hammack for a hike). SGOV 4 Nov sale no longer needed. || PREVIOUS ENTRY: Oct 28, 2026 - SGOV SLICE 1 BOOKED: SELL 100 at 100.6901 = 10,047.46 net (POEMS 1187938, 22:29 Bangkok). Cash 29,714.36; SGOV 694 sh parked (cost 69,917.06). || PREVIOUS ENTRY: Oct 28, 2026 13:16 Bangkok - PRICES OF THE 36 HOLDINGS SET TO THE TUE 2026-10-27 CLOSE FROM SALEE'S POEMS POSITIONS SCREEN (US market closed; POEMS "Current Price" column; SGOV mark 100.68). Reason: every web source reachable from the sandbox served pre-close cached pages for Oct 27 through both scheduled runs (00:30 and 03:30 UTC) and manual checks at 03:30-04:50 UTC, so 0 of 63 could be written by the job. The 27 watch names (no position) stay at the 26 Oct close until the next successful run. Moves of 6%+ vs 26 Oct: CDNS +6.5%, ALAB +10.5%, CRDO +10.8%, RKLB +8.3% - consistent with the reported 27 Oct session (AMD +5.5%, AVGO +4%, MU +2.8%, chips rally). Positions and cost on the same screen reconcile to the board to the cent on all 36 lines (641,827.76 NASD + 247,167.89 NYSE incl. SGOV = 888,995.64). pe/ps/fpe/peg/pfcf rescaled with price per the 26 Oct rule. || PREVIOUS ENTRY: Oct 28, 2026 (runs 00:30 + 03:30 UTC) - DAILY PRICE REFRESH: BOTH overnight passes could not resolve the Tue 2026-10-27 close for any ticker. 03:30 pass sampled 14 stockanalysis.com quote/history pages: every capture predated the 4:00 PM close (freshest stamps 10:05-11:25 AM EDT Oct 27; some caches as old as May 2025), and Google Finance (Sep 24/25 caches), marketscreener (Sep 4) and ycharts (Oct 26 18:04 EDT) were equally stale. Per the leave-unchanged rule nothing was written: all 63 prices, mcaps, P/E block, SPY/QQQ and pxd stay at the Mon 2026-10-26 close (CGNX still 2026-10-23); no HISTORY row; risk_series ust10/spy 10-27 skipped (sources unreadable; ust10 2026-10-26 = 5.00 was already added by the 00:30 pass). Oct-26 baseline cross-checked against 9 history tables - all matched. Every number checked came from a tool call this session; the next scheduled pass retries.</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>809580.01</v>
+        <v>773664.09</v>
       </c>
     </row>
     <row r="6">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>81422.16</v>
+        <v>45506.24</v>
       </c>
     </row>
     <row r="7">
@@ -517,7 +517,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>+11.18%</t>
+          <t>+6.25%</t>
         </is>
       </c>
     </row>
@@ -675,16 +675,16 @@
         <v>274.0825806451613</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>283.82</v>
+        <v>279.84</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>61588.94</v>
+        <v>60725.27999999999</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>2113.019999999997</v>
+        <v>1249.359999999993</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.03552731929157207</v>
+        <v>0.02100614837063459</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>32.2446</v>
@@ -693,7 +693,7 @@
         <v>1917777.250032</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>2072467.831</v>
+        <v>2043405.672</v>
       </c>
     </row>
     <row r="3">
@@ -722,16 +722,16 @@
         <v>457.2834126984127</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>530.14</v>
+        <v>521.91</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>66797.64</v>
+        <v>65760.65999999999</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>9179.93</v>
+        <v>8142.94999999999</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.1593247978789855</v>
+        <v>0.1413272065134138</v>
       </c>
       <c r="K3" s="3" t="n">
         <v>32.0119</v>
@@ -740,7 +740,7 @@
         <v>1844452.370749</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>2247740.586</v>
+        <v>2212846.208999999</v>
       </c>
     </row>
     <row r="4">
@@ -769,16 +769,16 @@
         <v>232.5394736842105</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>243.79</v>
+        <v>240.35</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>50952.11</v>
+        <v>50233.15</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>2351.360000000001</v>
+        <v>1632.400000000001</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.04838114638148589</v>
+        <v>0.03358795903355404</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>32.3066</v>
@@ -787,7 +787,7 @@
         <v>1570124.98995</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>1714538.5015</v>
+        <v>1690345.4975</v>
       </c>
     </row>
     <row r="5">
@@ -816,16 +816,16 @@
         <v>659.6042580645161</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>624.52</v>
+        <v>614.99</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>48400.3</v>
+        <v>47661.725</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>-2719.030000000006</v>
+        <v>-3457.605000000003</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.05318985988274897</v>
+        <v>-0.06763791700712829</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>32.2596</v>
@@ -834,7 +834,7 @@
         <v>1649089.138068</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>1628670.095</v>
+        <v>1603817.04625</v>
       </c>
     </row>
     <row r="6">
@@ -863,16 +863,16 @@
         <v>190.9340707964602</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>213.66</v>
+        <v>204.64</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>96574.31999999999</v>
+        <v>92497.28</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>10272.12</v>
+        <v>6195.080000000002</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.1190250074737376</v>
+        <v>0.07178356982788391</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>32.084</v>
@@ -881,7 +881,7 @@
         <v>2768919.7848</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>3249725.868</v>
+        <v>3112533.472</v>
       </c>
     </row>
     <row r="7">
@@ -910,16 +910,16 @@
         <v>340.3975141242938</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>345</v>
+        <v>326.08</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>30532.5</v>
+        <v>28858.08</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>407.3199999999997</v>
+        <v>-1267.100000000002</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.01352091506175232</v>
+        <v>-0.0420611594685908</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>31.6503</v>
@@ -928,7 +928,7 @@
         <v>953470.9845540001</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1027418.625</v>
+        <v>971074.3919999999</v>
       </c>
     </row>
     <row r="8">
@@ -957,16 +957,16 @@
         <v>250.7130909090909</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>566.42</v>
+        <v>504.8</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>31153.1</v>
+        <v>27764</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>17363.88</v>
+        <v>13974.78</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>1.259235837850146</v>
+        <v>1.013456888787038</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>32.0515</v>
@@ -975,7 +975,7 @@
         <v>441965.1848299999</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>1048301.815</v>
+        <v>934258.6</v>
       </c>
     </row>
     <row r="9">
@@ -1004,16 +1004,16 @@
         <v>215.550890052356</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>218.34</v>
+        <v>196.4</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>20851.47</v>
+        <v>18756.2</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>266.3600000000006</v>
+        <v>-1828.91</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.01293944992278402</v>
+        <v>-0.08884625829057993</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>32.5019</v>
@@ -1022,7 +1022,7 @@
         <v>669055.186709</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>701651.9655</v>
+        <v>631146.13</v>
       </c>
     </row>
     <row r="10">
@@ -1051,16 +1051,16 @@
         <v>326.5008333333333</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>342.75</v>
+        <v>327.89</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>4113</v>
+        <v>3934.68</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>194.9899999999998</v>
+        <v>16.66999999999962</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.04976761161916375</v>
+        <v>0.004254710937440082</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>32.32</v>
@@ -1069,7 +1069,7 @@
         <v>126630.0832</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>138402.45</v>
+        <v>132401.982</v>
       </c>
     </row>
     <row r="11">
@@ -1098,16 +1098,16 @@
         <v>378.1683870967742</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>431.81</v>
+        <v>406.13</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>73623.605</v>
+        <v>69245.16499999999</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>9145.894999999997</v>
+        <v>4767.454999999994</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.1418458409890797</v>
+        <v>0.07393958315206905</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>31.9974</v>
@@ -1116,7 +1116,7 @@
         <v>2063119.077954</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>2477434.30825</v>
+        <v>2330099.80225</v>
       </c>
     </row>
     <row r="12">
@@ -1145,16 +1145,16 @@
         <v>1345.164705882353</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>1675.7</v>
+        <v>1565.9</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>28486.9</v>
+        <v>26620.3</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>5619.100000000002</v>
+        <v>3752.500000000004</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.2457210575569142</v>
+        <v>0.1640953655358191</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>32.372</v>
@@ -1163,7 +1163,7 @@
         <v>740276.4216</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>958584.1850000001</v>
+        <v>895773.0950000001</v>
       </c>
     </row>
     <row r="13">
@@ -1192,16 +1192,16 @@
         <v>186.3690909090909</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>254.39</v>
+        <v>239.11</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>5596.58</v>
+        <v>5260.42</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>1496.46</v>
+        <v>1160.3</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.3649795615738076</v>
+        <v>0.2829917173155908</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>31.4491</v>
@@ -1210,7 +1210,7 @@
         <v>128945.083892</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>188324.917</v>
+        <v>177013.133</v>
       </c>
     </row>
     <row r="14">
@@ -1239,16 +1239,16 @@
         <v>345.6519298245614</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>421.66</v>
+        <v>390.09</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>24034.62</v>
+        <v>22235.13</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4332.460000000003</v>
+        <v>2532.969999999998</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>0.2198977167985643</v>
+        <v>0.1285630611059903</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>32.1085</v>
@@ -1257,7 +1257,7 @@
         <v>632606.80436</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>808764.9630000001</v>
+        <v>748212.1244999999</v>
       </c>
     </row>
     <row r="15">
@@ -1286,16 +1286,16 @@
         <v>195.0383333333333</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>167.43</v>
+        <v>157.91</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>3013.74</v>
+        <v>2842.38</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>-496.9499999999998</v>
+        <v>-668.3099999999999</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.1415533698503712</v>
+        <v>-0.1903642873623134</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>32.1216</v>
@@ -1304,7 +1304,7 @@
         <v>112768.979904</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>101412.351</v>
+        <v>95646.087</v>
       </c>
     </row>
     <row r="16">
@@ -1333,16 +1333,16 @@
         <v>356.737</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>296.23</v>
+        <v>274.37</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>2962.3</v>
+        <v>2743.7</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-605.0699999999997</v>
+        <v>-823.6700000000001</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.1696123474716667</v>
+        <v>-0.2308899833771098</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>32.6972</v>
@@ -1351,7 +1351,7 @@
         <v>116643.010364</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>99681.395</v>
+        <v>92325.50499999999</v>
       </c>
     </row>
     <row r="17">
@@ -1380,16 +1380,16 @@
         <v>753.9935288169869</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>934.27</v>
+        <v>884.74</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>46199.6515</v>
+        <v>43750.393</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>8914.671499999997</v>
+        <v>6465.413</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.2390955151377309</v>
+        <v>0.1734052961809286</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>32.1376</v>
@@ -1398,7 +1398,7 @@
         <v>1198249.773248</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>1554618.272975</v>
+        <v>1472200.72445</v>
       </c>
     </row>
     <row r="18">
@@ -1427,16 +1427,16 @@
         <v>159.0364285714286</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>184.22</v>
+        <v>168.86</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>18053.56</v>
+        <v>16548.28</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>2467.990000000002</v>
+        <v>962.7100000000028</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.15835096181917</v>
+        <v>0.0617693161045764</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>32.6011</v>
@@ -1445,7 +1445,7 @@
         <v>508106.726127</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>607502.294</v>
+        <v>556849.6220000001</v>
       </c>
     </row>
     <row r="19">
@@ -1474,16 +1474,16 @@
         <v>79.426</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>82.08</v>
+        <v>79.3</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>8618.4</v>
+        <v>8326.5</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>278.6700000000001</v>
+        <v>-13.22999999999956</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.03341475083725733</v>
+        <v>-0.001586382292951878</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>32.34</v>
@@ -1492,7 +1492,7 @@
         <v>269706.8682</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>290009.16</v>
+        <v>280186.725</v>
       </c>
     </row>
     <row r="20">
@@ -1521,16 +1521,16 @@
         <v>815.0208695652174</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>919.53</v>
+        <v>840.7</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>10574.595</v>
+        <v>9668.050000000001</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>1201.855</v>
+        <v>295.3100000000013</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.1282287783508344</v>
+        <v>0.03150732870003876</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>32.5803</v>
@@ -1539,7 +1539,7 @@
         <v>305366.681022</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>355835.12175</v>
+        <v>325329.8825</v>
       </c>
     </row>
     <row r="21">
@@ -1568,16 +1568,16 @@
         <v>253.698</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>290.43</v>
+        <v>258.7</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>4356.45</v>
+        <v>3880.5</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>550.98</v>
+        <v>75.0300000000002</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.1447863207435613</v>
+        <v>0.01971635566697417</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>32.4697</v>
@@ -1586,7 +1586,7 @@
         <v>123562.469259</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>146594.5425</v>
+        <v>130578.825</v>
       </c>
     </row>
     <row r="22">
@@ -1615,16 +1615,16 @@
         <v>157.2364864864865</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>165.29</v>
+        <v>150.99</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>18347.19</v>
+        <v>16759.89</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>893.9399999999987</v>
+        <v>-693.3600000000006</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.05121911391861107</v>
+        <v>-0.0397266984659018</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>32.4342</v>
@@ -1633,7 +1633,7 @@
         <v>566082.20115</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>617382.9434999999</v>
+        <v>563970.2984999999</v>
       </c>
     </row>
     <row r="23">
@@ -1662,16 +1662,16 @@
         <v>200.356</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>176.89</v>
+        <v>174.4</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1768.9</v>
+        <v>1744</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>-234.6600000000001</v>
+        <v>-259.5599999999999</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.1171215236878357</v>
+        <v>-0.1295494020643255</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>33.65</v>
@@ -1680,7 +1680,7 @@
         <v>67419.79399999999</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>59523.48499999999</v>
+        <v>58685.6</v>
       </c>
     </row>
     <row r="24">
@@ -1709,16 +1709,16 @@
         <v>65.60677419354839</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>58.97</v>
+        <v>56.15</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>3656.14</v>
+        <v>3481.3</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>-411.48</v>
+        <v>-586.3200000000002</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>-0.1011598920253121</v>
+        <v>-0.1441432582197944</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>33.0687</v>
@@ -1727,7 +1727,7 @@
         <v>134510.905494</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>123029.111</v>
+        <v>117145.745</v>
       </c>
     </row>
     <row r="25">
@@ -1756,16 +1756,16 @@
         <v>84.45999999999999</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>59.1</v>
+        <v>54.73</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1359.3</v>
+        <v>1258.79</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-583.28</v>
+        <v>-683.79</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>-0.3002604783329387</v>
+        <v>-0.3520009471939379</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>33.31</v>
@@ -1774,7 +1774,7 @@
         <v>64707.3398</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>45740.445</v>
+        <v>42358.2835</v>
       </c>
     </row>
     <row r="26">
@@ -1803,16 +1803,16 @@
         <v>138.32725</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>196.42</v>
+        <v>184.11</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>7856.799999999999</v>
+        <v>7364.400000000001</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>2323.709999999999</v>
+        <v>1831.31</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>0.4199660587483665</v>
+        <v>0.3309741934434467</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>31.79</v>
@@ -1821,7 +1821,7 @@
         <v>175896.9311</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>264381.3199999999</v>
+        <v>247812.06</v>
       </c>
     </row>
     <row r="27">
@@ -1850,16 +1850,16 @@
         <v>208.7944444444445</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>134.88</v>
+        <v>126.11</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>2427.84</v>
+        <v>2269.98</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-1330.46</v>
+        <v>-1488.32</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>-0.3540058004949046</v>
+        <v>-0.3960088337812309</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>32.3497</v>
@@ -1868,7 +1868,7 @@
         <v>121579.87751</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>81696.81600000001</v>
+        <v>76384.82699999999</v>
       </c>
     </row>
     <row r="28">
@@ -1897,16 +1897,16 @@
         <v>431.0968421052632</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>448.76</v>
+        <v>432.01</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>17052.88</v>
+        <v>16416.38</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>671.2000000000007</v>
+        <v>34.70000000000073</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>0.04097259865898984</v>
+        <v>0.002118219865117663</v>
       </c>
       <c r="K28" s="3" t="n">
         <v>32.1878</v>
@@ -1915,7 +1915,7 @@
         <v>527290.2395040001</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>573829.412</v>
+        <v>552411.187</v>
       </c>
     </row>
     <row r="29">
@@ -1944,16 +1944,16 @@
         <v>376.0583333333333</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>410.54</v>
+        <v>413.59</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>7389.72</v>
+        <v>7444.62</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>620.6700000000001</v>
+        <v>675.5699999999997</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.0916923349657633</v>
+        <v>0.0998027788242072</v>
       </c>
       <c r="K29" s="3" t="n">
         <v>33.65</v>
@@ -1962,7 +1962,7 @@
         <v>227778.5325</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>248664.078</v>
+        <v>250511.463</v>
       </c>
     </row>
     <row r="30">
@@ -1991,16 +1991,16 @@
         <v>249.8636842105263</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>380.57</v>
+        <v>365.87</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>14461.66</v>
+        <v>13903.06</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>4966.84</v>
+        <v>4408.24</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.5231104960388928</v>
+        <v>0.4642784170737307</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>32.5467</v>
@@ -2009,7 +2009,7 @@
         <v>309025.058094</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>486634.859</v>
+        <v>467837.969</v>
       </c>
     </row>
     <row r="31">
@@ -2038,16 +2038,16 @@
         <v>960.0600000000001</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>887.85</v>
+        <v>857.87</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>11542.05</v>
+        <v>11152.31</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-938.7299999999996</v>
+        <v>-1328.470000000001</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>-0.07521404912192985</v>
+        <v>-0.1064412640876613</v>
       </c>
       <c r="K31" s="3" t="n">
         <v>32.66</v>
@@ -2056,7 +2056,7 @@
         <v>407622.2748</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>388389.9825</v>
+        <v>375275.2315</v>
       </c>
     </row>
     <row r="32">
@@ -2085,16 +2085,16 @@
         <v>418.511923076923</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>393.72</v>
+        <v>369.97</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>10236.72</v>
+        <v>9619.220000000001</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-644.5899999999983</v>
+        <v>-1262.089999999998</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>-0.05923827186248699</v>
+        <v>-0.1159869537767051</v>
       </c>
       <c r="K32" s="3" t="n">
         <v>32.3317</v>
@@ -2103,7 +2103,7 @@
         <v>351811.2505269999</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>344465.628</v>
+        <v>323686.753</v>
       </c>
     </row>
     <row r="33">
@@ -2132,16 +2132,16 @@
         <v>246.5205952380952</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>245.92</v>
+        <v>232.5</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>20657.28</v>
+        <v>19530</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>-50.45000000000073</v>
+        <v>-1177.73</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>-0.002436288284616456</v>
+        <v>-0.05687393065294939</v>
       </c>
       <c r="K33" s="3" t="n">
         <v>31.4889</v>
@@ -2150,7 +2150,7 @@
         <v>652063.639197</v>
       </c>
       <c r="M33" s="6" t="n">
-        <v>695117.472</v>
+        <v>657184.5</v>
       </c>
     </row>
     <row r="34">
@@ -2179,16 +2179,16 @@
         <v>263.88640625</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>264.58</v>
+        <v>262.38</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>16933.12</v>
+        <v>16792.32</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>44.38999999999942</v>
+        <v>-96.40999999999985</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.002628379990680141</v>
+        <v>-0.005708540547453826</v>
       </c>
       <c r="K34" s="3" t="n">
         <v>33.0112</v>
@@ -2197,7 +2197,7 @@
         <v>557517.243776</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>569799.4879999999</v>
+        <v>565061.568</v>
       </c>
     </row>
     <row r="35">
@@ -2226,16 +2226,16 @@
         <v>140.3488679245283</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>140.95</v>
+        <v>138.37</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>14940.7</v>
+        <v>14667.22</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>63.71999999999935</v>
+        <v>-209.7599999999984</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>0.004283127355148649</v>
+        <v>-0.01409963581318241</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>32.9329</v>
@@ -2244,7 +2244,7 @@
         <v>489942.0946419999</v>
       </c>
       <c r="M35" s="6" t="n">
-        <v>502754.5549999999</v>
+        <v>493551.953</v>
       </c>
     </row>
     <row r="36">
@@ -2273,16 +2273,16 @@
         <v>248.6436956521739</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>348.91</v>
+        <v>344.63</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>16049.86</v>
+        <v>15852.98</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>4612.25</v>
+        <v>4415.369999999999</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.4032529523213328</v>
+        <v>0.3860395659582727</v>
       </c>
       <c r="K36" s="3" t="n">
         <v>32.4331</v>
@@ -2291,7 +2291,7 @@
         <v>370957.1488910001</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>540077.789</v>
+        <v>533452.777</v>
       </c>
     </row>
     <row r="37">
@@ -2320,16 +2320,16 @@
         <v>717.9223076923076</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>647.39</v>
+        <v>622.75</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>8416.07</v>
+        <v>8095.75</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>-916.9200000000001</v>
+        <v>-1237.24</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>-0.09824504258549512</v>
+        <v>-0.1325663051176525</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>33.65</v>
@@ -2338,7 +2338,7 @@
         <v>314055.1135</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>283200.7555</v>
+        <v>272421.9875</v>
       </c>
     </row>
     <row r="38">
@@ -2351,13 +2351,13 @@
         <v>728157.85</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>809580.0115</v>
+        <v>773664.093</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>81422.16150000005</v>
+        <v>45506.24300000002</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>0.1118193829813138</v>
+        <v>0.06249502494548403</v>
       </c>
     </row>
   </sheetData>
@@ -2552,22 +2552,22 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>283.82</v>
+        <v>279.84</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3474.73</v>
+        <v>3426.004</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>14.82</v>
+        <v>14.61</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>21.22</v>
+        <v>20.92</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>7.38</v>
+        <v>7.28</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1.59</v>
+        <v>1.57</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>60.86</v>
@@ -2639,22 +2639,22 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>530.14</v>
+        <v>521.91</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>3948.9209</v>
+        <v>3887.6171</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>27.68</v>
+        <v>27.25</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>26.83</v>
+        <v>26.41</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>11.4</v>
+        <v>11.22</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.69</v>
+        <v>1.66</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>67.66</v>
@@ -2726,22 +2726,22 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>243.79</v>
+        <v>240.35</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2630.18</v>
+        <v>2593.0668</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>28.31</v>
+        <v>27.91</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>25.95</v>
+        <v>25.58</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>3.39</v>
+        <v>3.34</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.25</v>
+        <v>1.23</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>50.77</v>
@@ -2810,22 +2810,22 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>624.52</v>
+        <v>614.99</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1595.0783</v>
+        <v>1570.7379</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>21.3</v>
+        <v>20.97</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>18.97</v>
+        <v>18.68</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>81.03</v>
@@ -2897,22 +2897,22 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>213.66</v>
+        <v>204.64</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5172.6056</v>
+        <v>4954.2357</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>27.01</v>
+        <v>25.87</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>17.67</v>
+        <v>16.92</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>17.07</v>
+        <v>16.35</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>75</v>
@@ -2984,22 +2984,22 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>345</v>
+        <v>326.08</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1639.566</v>
+        <v>1549.6513</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>44.01</v>
+        <v>41.6</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>19.87</v>
+        <v>18.78</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>18.4</v>
+        <v>17.39</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>68.77</v>
@@ -3071,22 +3071,22 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>566.42</v>
+        <v>504.8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>924.6671</v>
+        <v>824.0739</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>145.61</v>
+        <v>129.77</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>50.96</v>
+        <v>45.42</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>22.39</v>
+        <v>19.95</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.77</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>53.06</v>
@@ -3158,22 +3158,22 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>228.77</v>
+        <v>205.97</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>244.3489</v>
+        <v>219.9963</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>233.44</v>
+        <v>210.17</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>95.79000000000001</v>
+        <v>86.23999999999999</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>47.35</v>
+        <v>42.63</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3.15</v>
+        <v>2.84</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>97.54000000000001</v>
@@ -3245,22 +3245,22 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>218.34</v>
+        <v>196.4</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>191.2133</v>
+        <v>171.9991</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>72.78</v>
+        <v>65.47</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>38.64</v>
+        <v>34.76</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>20.23</v>
+        <v>18.2</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.62</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>53.1</v>
@@ -3329,22 +3329,22 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>342.75</v>
+        <v>327.89</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>94.51000000000001</v>
+        <v>90.41249999999999</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>68.14</v>
+        <v>65.19</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>39.84</v>
+        <v>38.11</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>15.42</v>
+        <v>14.75</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>2.64</v>
+        <v>2.53</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>85.68000000000001</v>
@@ -3416,22 +3416,22 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>490.19</v>
+        <v>467.61</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>93.8633</v>
+        <v>89.53959999999999</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>86.61</v>
+        <v>82.62</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>27.75</v>
+        <v>26.47</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>9.960000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>72.59999999999999</v>
@@ -3503,22 +3503,22 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1198.81</v>
+        <v>1211.63</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>58.9167</v>
+        <v>59.5468</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>73.14</v>
+        <v>73.92</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>37.1</v>
+        <v>37.5</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>18.02</v>
+        <v>18.21</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>55.2</v>
@@ -3590,19 +3590,19 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>431.81</v>
+        <v>406.13</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>2082.9404</v>
+        <v>1959.0667</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>28.56</v>
+        <v>26.86</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>20.22</v>
+        <v>19.02</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>13.6</v>
+        <v>12.79</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>65.83</v>
@@ -3674,19 +3674,19 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1675.7</v>
+        <v>1565.9</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>654.365</v>
+        <v>611.4878</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>42.7</v>
+        <v>39.9</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>26.37</v>
+        <v>24.64</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>14.8</v>
+        <v>13.83</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>54.34</v>
@@ -3758,22 +3758,22 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>254.39</v>
+        <v>239.11</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>318.3134</v>
+        <v>299.1938</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>37.91</v>
+        <v>35.63</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>24.76</v>
+        <v>23.27</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>12.18</v>
+        <v>11.45</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>51.05</v>
@@ -3845,22 +3845,22 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>421.66</v>
+        <v>390.09</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>334.783</v>
+        <v>309.7175</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>36.35</v>
+        <v>33.63</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>23.91</v>
+        <v>22.12</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>10.86</v>
+        <v>10.05</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>50.3</v>
@@ -3932,22 +3932,22 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>167.43</v>
+        <v>157.91</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>218.7082</v>
+        <v>206.2725</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>41.96</v>
+        <v>39.57</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>30.65</v>
+        <v>28.91</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>15.07</v>
+        <v>14.21</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1.52</v>
+        <v>1.43</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>61.3</v>
@@ -4019,22 +4019,22 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>296.23</v>
+        <v>274.37</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46.6535</v>
+        <v>43.2108</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>34.01</v>
+        <v>31.5</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>31.77</v>
+        <v>29.43</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>9.33</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.87</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>59.3</v>
@@ -4106,19 +4106,19 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>934.27</v>
+        <v>884.74</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1055.1562</v>
+        <v>999.2175</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>12.57</v>
+        <v>11.9</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>5.29</v>
+        <v>5.01</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>7.92</v>
+        <v>7.5</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>0.07000000000000001</v>
@@ -4193,22 +4193,22 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1330.05</v>
+        <v>1150.89</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>196.9623</v>
+        <v>170.4311</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>18.03</v>
+        <v>15.6</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>6.18</v>
+        <v>5.35</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>9.73</v>
+        <v>8.42</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>71.47</v>
@@ -4277,22 +4277,22 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>700.47</v>
+        <v>644.58</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>158.492</v>
+        <v>145.846</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>36.75</v>
+        <v>33.82</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>20.05</v>
+        <v>18.45</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>11.48</v>
+        <v>10.56</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>50.3</v>
@@ -4364,22 +4364,22 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>184.22</v>
+        <v>168.86</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>230.462</v>
+        <v>211.2464</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>58.3</v>
+        <v>53.44</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>39.61</v>
+        <v>36.31</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>21.86</v>
+        <v>20.04</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1.58</v>
+        <v>1.45</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>63.54</v>
@@ -4448,22 +4448,22 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>82.08</v>
+        <v>79.3</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>202.4112</v>
+        <v>195.5557</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>29.63</v>
+        <v>28.63</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>27.58</v>
+        <v>26.65</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>6.13</v>
+        <v>5.92</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>38.81</v>
@@ -4535,22 +4535,22 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>128.87</v>
+        <v>123.31</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>111.0123</v>
+        <v>106.2228</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>52.6</v>
+        <v>50.33</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>34.27</v>
+        <v>32.79</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>6.26</v>
+        <v>5.99</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1.07</v>
+        <v>1.02</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>36.5</v>
@@ -4622,19 +4622,19 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>919.53</v>
+        <v>840.7</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>71.533</v>
+        <v>65.4006</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>42.21</v>
+        <v>38.59</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>23.77</v>
+        <v>21.73</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.36</v>
+        <v>0.33</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>41.7</v>
@@ -4703,22 +4703,22 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>236.9</v>
+        <v>210.32</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46.3437</v>
+        <v>41.144</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>57.5</v>
+        <v>51.05</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>25.24</v>
+        <v>22.41</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>6.51</v>
+        <v>5.78</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.47</v>
+        <v>0.42</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>37.5</v>
@@ -4784,22 +4784,22 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>290.43</v>
+        <v>258.7</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>49.7817</v>
+        <v>44.343</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>165.02</v>
+        <v>146.99</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>51.69</v>
+        <v>46.04</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>41.48</v>
+        <v>36.95</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0.98</v>
+        <v>0.87</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>75.98999999999999</v>
@@ -4871,22 +4871,22 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>165.29</v>
+        <v>150.99</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>30.8247</v>
+        <v>28.1579</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>58.2</v>
+        <v>53.16</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>22.66</v>
+        <v>20.7</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>19.39</v>
+        <v>17.71</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.44</v>
+        <v>0.4</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>67.06999999999999</v>
@@ -4958,19 +4958,19 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>349.15</v>
+        <v>327.29</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>12.5131</v>
+        <v>11.7297</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>26.75</v>
+        <v>25.08</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>19.14</v>
+        <v>17.94</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>2.7</v>
+        <v>2.53</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>12</v>
@@ -5039,22 +5039,22 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>176.89</v>
+        <v>174.4</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>19.0437</v>
+        <v>18.7756</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>10.91</v>
+        <v>10.76</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>8.4</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>3.54</v>
+        <v>3.49</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>44.02</v>
@@ -5126,19 +5126,19 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>58.97</v>
+        <v>56.15</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>9.819599999999999</v>
+        <v>9.35</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>57.25</v>
+        <v>54.51</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>32.87</v>
+        <v>31.3</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>9.02</v>
+        <v>8.59</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>68.87</v>
@@ -5210,16 +5210,16 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>143.89</v>
+        <v>134.72</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>1952.5843</v>
+        <v>1828.1476</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>51.04</v>
+        <v>47.79</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>60.94</v>
+        <v>57.06</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>51.87</v>
@@ -5276,13 +5276,13 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>59.1</v>
+        <v>54.73</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>35.3688</v>
+        <v>32.7535</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>45.98</v>
+        <v>42.58</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>37.27</v>
@@ -5345,22 +5345,22 @@
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>196.42</v>
+        <v>184.11</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>470.8766</v>
+        <v>441.3659</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>167.88</v>
+        <v>157.36</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>103.24</v>
+        <v>96.77</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>76.56999999999999</v>
+        <v>71.77</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>1.94</v>
+        <v>1.82</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>84.06999999999999</v>
@@ -5432,22 +5432,22 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>279.12</v>
+        <v>277.61</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>51.9764</v>
+        <v>51.6952</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>28.19</v>
+        <v>28.04</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>22.17</v>
+        <v>22.05</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>2.27</v>
+        <v>2.26</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1.33</v>
+        <v>1.32</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>25.48</v>
@@ -5513,19 +5513,19 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>43.59</v>
+        <v>41.09</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>8.180999999999999</v>
+        <v>7.7118</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>256.41</v>
+        <v>241.7</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>46.05</v>
+        <v>43.41</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>5.38</v>
+        <v>5.07</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>23</v>
@@ -5594,19 +5594,19 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>134.88</v>
+        <v>126.11</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>6.7958</v>
+        <v>6.3539</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>40.22</v>
+        <v>37.6</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>3.4</v>
+        <v>3.18</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>1.19</v>
+        <v>1.11</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>26.47</v>
@@ -5672,22 +5672,22 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>265.84</v>
+        <v>235.27</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>94.6082</v>
+        <v>83.72880000000001</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>531.6799999999999</v>
+        <v>470.54</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>100.25</v>
+        <v>88.72</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>23.83</v>
+        <v>21.09</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>4.04</v>
+        <v>3.58</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>79.53</v>
@@ -5756,22 +5756,22 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>448.76</v>
+        <v>432.01</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>158.5321</v>
+        <v>152.6149</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>54.26</v>
+        <v>52.23</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>37.25</v>
+        <v>35.86</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>13.69</v>
+        <v>13.18</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>2.38</v>
+        <v>2.29</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>67.19</v>
@@ -5840,22 +5840,22 @@
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>139.51</v>
+        <v>130.67</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>421.8443</v>
+        <v>395.1143</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>21.87</v>
+        <v>20.48</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>16.39</v>
+        <v>15.35</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5.88</v>
+        <v>5.51</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>63.96</v>
@@ -5924,22 +5924,22 @@
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>410.54</v>
+        <v>413.59</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>753.5944</v>
+        <v>759.193</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>33.32</v>
+        <v>33.57</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>28.17</v>
+        <v>28.38</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>16.42</v>
+        <v>16.54</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>1.95</v>
+        <v>1.96</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>80.18000000000001</v>
@@ -6011,22 +6011,22 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>91.59</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>82.4657</v>
+        <v>76.5232</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>42.4</v>
+        <v>39.34</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>36.84</v>
+        <v>34.19</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>16.23</v>
+        <v>15.06</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
       <c r="I43" s="3" t="n">
         <v>92.23999999999999</v>
@@ -6098,22 +6098,22 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>380.57</v>
+        <v>365.87</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>311.3035</v>
+        <v>299.279</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>951.42</v>
+        <v>914.67</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>90.8</v>
+        <v>87.29000000000001</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>27.12</v>
+        <v>26.07</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>4.84</v>
+        <v>4.65</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>70.36</v>
@@ -6185,22 +6185,22 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>261.15</v>
+        <v>250.43</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>267.9734</v>
+        <v>256.9733</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>6528.75</v>
+        <v>6260.75</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>184.86</v>
+        <v>177.27</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>49.72</v>
+        <v>47.68</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>6.31</v>
+        <v>6.05</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>75.14</v>
@@ -6266,22 +6266,22 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>139.1</v>
+        <v>136.08</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>101.9067</v>
+        <v>99.6942</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>45.31</v>
+        <v>44.33</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>39.62</v>
+        <v>38.76</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>12.93</v>
+        <v>12.65</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>2.42</v>
+        <v>2.37</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>79.75</v>
@@ -6353,19 +6353,19 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>310.04</v>
+        <v>280.7</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>110.0499</v>
+        <v>99.6356</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>209.32</v>
+        <v>189.51</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>43.84</v>
+        <v>39.69</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>72.58</v>
@@ -6431,22 +6431,22 @@
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>137.98</v>
+        <v>130.7</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>12.7665</v>
+        <v>12.0929</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>35.75</v>
+        <v>33.86</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>27.69</v>
+        <v>26.23</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>3.64</v>
+        <v>3.45</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>2.09</v>
+        <v>1.98</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>22.08</v>
@@ -6518,22 +6518,22 @@
         </is>
       </c>
       <c r="C49" s="3" t="n">
-        <v>887.85</v>
+        <v>857.87</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>236.4606</v>
+        <v>228.476</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>23.24</v>
+        <v>22.46</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>42.27</v>
+        <v>40.84</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>5.37</v>
+        <v>5.19</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="I49" s="3" t="n">
         <v>20.57</v>
@@ -6605,22 +6605,22 @@
         </is>
       </c>
       <c r="C50" s="3" t="n">
-        <v>393.72</v>
+        <v>369.97</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>152.877</v>
+        <v>143.6551</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>40.09</v>
+        <v>37.67</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>25.98</v>
+        <v>24.41</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>5.09</v>
+        <v>4.78</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>1.97</v>
+        <v>1.85</v>
       </c>
       <c r="I50" s="3" t="n">
         <v>36.1</v>
@@ -6692,22 +6692,22 @@
         </is>
       </c>
       <c r="C51" s="3" t="n">
-        <v>245.92</v>
+        <v>232.5</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>94.6756</v>
+        <v>89.5091</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>45.96</v>
+        <v>43.45</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>31.05</v>
+        <v>29.36</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>7.21</v>
+        <v>6.82</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>0.78</v>
+        <v>0.74</v>
       </c>
       <c r="I51" s="3" t="n">
         <v>38.12</v>
@@ -6779,22 +6779,22 @@
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>632.79</v>
+        <v>620.73</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>95.13760000000001</v>
+        <v>93.3244</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>72.40000000000001</v>
+        <v>71.02</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>34.04</v>
+        <v>33.39</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>2.89</v>
+        <v>2.83</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>1.64</v>
+        <v>1.61</v>
       </c>
       <c r="I52" s="3" t="n">
         <v>15.46</v>
@@ -6866,22 +6866,22 @@
         </is>
       </c>
       <c r="C53" s="3" t="n">
-        <v>222.28</v>
+        <v>203.17</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>65.4663</v>
+        <v>59.838</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>129.23</v>
+        <v>118.12</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>45.89</v>
+        <v>41.94</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>17.09</v>
+        <v>15.62</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>0.49</v>
+        <v>0.45</v>
       </c>
       <c r="I53" s="3" t="n">
         <v>32.66</v>
@@ -6950,22 +6950,22 @@
         </is>
       </c>
       <c r="C54" s="3" t="n">
-        <v>264.58</v>
+        <v>262.38</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>94.4799</v>
+        <v>93.6943</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>25.61</v>
+        <v>25.4</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>21.39</v>
+        <v>21.21</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>3.02</v>
+        <v>2.99</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="I54" s="3" t="n">
         <v>22.11</v>
@@ -7037,22 +7037,22 @@
         </is>
       </c>
       <c r="C55" s="3" t="n">
-        <v>140.95</v>
+        <v>138.37</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>47.5258</v>
+        <v>46.6559</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>24.01</v>
+        <v>23.57</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>13.89</v>
+        <v>13.64</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="I55" s="3" t="n">
         <v>38.31</v>
@@ -7124,22 +7124,22 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>348.91</v>
+        <v>344.63</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>5093.9916</v>
+        <v>5031.5048</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>39.83</v>
+        <v>39.34</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>38.05</v>
+        <v>37.58</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>10.91</v>
+        <v>10.78</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>3.43</v>
+        <v>3.39</v>
       </c>
       <c r="I56" s="3" t="n">
         <v>48.65</v>
@@ -7211,16 +7211,16 @@
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>62.05</v>
+        <v>62.08</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>258.3684</v>
+        <v>258.4933</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>17.99</v>
+        <v>18</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>17.29</v>
+        <v>17.3</v>
       </c>
       <c r="G57" s="3" t="n">
         <v>5.2</v>
@@ -7298,22 +7298,22 @@
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>254.91</v>
+        <v>228.5</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>85.6374</v>
+        <v>76.7649</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>19.59</v>
+        <v>17.56</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>14.19</v>
+        <v>12.72</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>12.54</v>
+        <v>11.24</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
       <c r="I58" s="3" t="n">
         <v>88.45999999999999</v>
@@ -7382,22 +7382,22 @@
         </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>76.58</v>
+        <v>74.23999999999999</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46.9057</v>
+        <v>45.4724</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>29.57</v>
+        <v>28.67</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>17.99</v>
+        <v>17.44</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>1.69</v>
+        <v>1.64</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="I59" s="3" t="n">
         <v>44.34</v>
@@ -7469,22 +7469,22 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>647.39</v>
+        <v>622.75</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>297.586</v>
+        <v>286.2597</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>27.9</v>
+        <v>26.84</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>22.34</v>
+        <v>21.49</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>3.98</v>
+        <v>3.83</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>1.22</v>
+        <v>1.17</v>
       </c>
       <c r="I60" s="3" t="n">
         <v>29.71</v>
@@ -7556,22 +7556,22 @@
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>313.28</v>
+        <v>301.8</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>325.0469</v>
+        <v>313.1357</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>36.13</v>
+        <v>34.81</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>35.26</v>
+        <v>33.97</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>6.18</v>
+        <v>5.95</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>2.25</v>
+        <v>2.17</v>
       </c>
       <c r="I61" s="3" t="n">
         <v>30.07</v>
@@ -7643,22 +7643,22 @@
         </is>
       </c>
       <c r="C62" s="3" t="n">
-        <v>373.66</v>
+        <v>345.91</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>11.4272</v>
+        <v>10.5786</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>20.97</v>
+        <v>19.41</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>16.64</v>
+        <v>15.4</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>2.65</v>
+        <v>2.45</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>0.41</v>
+        <v>0.38</v>
       </c>
       <c r="I62" s="3" t="n">
         <v>23.78</v>
@@ -7730,22 +7730,22 @@
         </is>
       </c>
       <c r="C63" s="3" t="n">
-        <v>187.92</v>
+        <v>166.48</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>21.2421</v>
+        <v>18.8186</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>74.28</v>
+        <v>65.81</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>36.41</v>
+        <v>32.26</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>12.42</v>
+        <v>11</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>0.84</v>
+        <v>0.74</v>
       </c>
       <c r="I63" s="3" t="n">
         <v>26.87</v>
@@ -7814,22 +7814,22 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>348.57</v>
+        <v>320.72</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>49.4324</v>
+        <v>45.4829</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>77.98</v>
+        <v>71.75</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>33.49</v>
+        <v>30.81</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>8.210000000000001</v>
+        <v>7.55</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>0.46</v>
+        <v>0.42</v>
       </c>
       <c r="I64" s="3" t="n">
         <v>44.07</v>

</xml_diff>